<commit_message>
Seprated SNG and added quinoa and sweet lupin crops
</commit_message>
<xml_diff>
--- a/data/default/CropProduction.xlsx
+++ b/data/default/CropProduction.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="179">
   <si>
     <t>f_crop</t>
   </si>
@@ -567,6 +567,21 @@
   <si>
     <t>Ahlgren et al (2022)</t>
   </si>
+  <si>
+    <t>Semi-natural pastures, thin soils</t>
+  </si>
+  <si>
+    <t>Semi-natural pastures, wooded</t>
+  </si>
+  <si>
+    <t>Quinoa</t>
+  </si>
+  <si>
+    <t>assumed same as dry peas</t>
+  </si>
+  <si>
+    <t>Sweet lupin</t>
+  </si>
 </sst>
 </file>
 
@@ -575,7 +590,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -628,6 +643,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="7"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -656,7 +678,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -670,6 +692,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -951,7 +974,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I215"/>
+  <dimension ref="A1:I223"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="30.42578125" customWidth="1"/>
@@ -1479,255 +1502,265 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>35</v>
+        <v>174</v>
       </c>
       <c r="B31" s="3"/>
       <c r="D31" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E31" t="s">
         <v>47</v>
       </c>
       <c r="F31">
-        <v>1</v>
+        <v>0.45</v>
       </c>
       <c r="G31" t="s">
         <v>155</v>
       </c>
+      <c r="H31" s="4"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="A32" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B32" s="3"/>
+      <c r="D32" t="s">
+        <v>46</v>
+      </c>
+      <c r="E32" t="s">
+        <v>47</v>
+      </c>
+      <c r="F32">
+        <v>0.45</v>
+      </c>
+      <c r="G32" t="s">
+        <v>155</v>
+      </c>
+      <c r="H32" s="4"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="3"/>
+      <c r="D33" t="s">
+        <v>43</v>
+      </c>
+      <c r="E33" t="s">
+        <v>47</v>
+      </c>
+      <c r="F33">
+        <v>1</v>
+      </c>
+      <c r="G33" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>58</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D34" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="E32" t="s">
-        <v>47</v>
-      </c>
-      <c r="F32">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="E34" t="s">
+        <v>47</v>
+      </c>
+      <c r="F34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>50</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D35" t="s">
         <v>86</v>
       </c>
-      <c r="E33" t="s">
-        <v>47</v>
-      </c>
-      <c r="F33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
+      <c r="E35" t="s">
+        <v>47</v>
+      </c>
+      <c r="F35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B34" s="4"/>
-      <c r="D34" s="4" t="s">
+      <c r="B36" s="4"/>
+      <c r="D36" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="E34" t="s">
-        <v>47</v>
-      </c>
-      <c r="F34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+      <c r="E36" t="s">
+        <v>47</v>
+      </c>
+      <c r="F36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>21</v>
       </c>
-      <c r="D35" s="6" t="s">
+      <c r="D37" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="E35" t="s">
-        <v>47</v>
-      </c>
-      <c r="F35">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+      <c r="E37" t="s">
+        <v>47</v>
+      </c>
+      <c r="F37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>16</v>
       </c>
-      <c r="D36" s="6" t="s">
+      <c r="D38" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="E36" t="s">
-        <v>47</v>
-      </c>
-      <c r="F36">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+      <c r="E38" t="s">
+        <v>47</v>
+      </c>
+      <c r="F38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>51</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D39" t="s">
         <v>81</v>
       </c>
-      <c r="E37" t="s">
-        <v>47</v>
-      </c>
-      <c r="F37">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+      <c r="E39" t="s">
+        <v>47</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>65</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="D40" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E38" t="s">
-        <v>47</v>
-      </c>
-      <c r="F38">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
+      <c r="E40" t="s">
+        <v>47</v>
+      </c>
+      <c r="F40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B39" s="4"/>
-      <c r="D39" s="7" t="s">
+      <c r="B41" s="4"/>
+      <c r="D41" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="E39" t="s">
-        <v>47</v>
-      </c>
-      <c r="F39">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="s">
+      <c r="E41" t="s">
+        <v>47</v>
+      </c>
+      <c r="F41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B40" s="4"/>
-      <c r="D40" s="7" t="s">
+      <c r="B42" s="4"/>
+      <c r="D42" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="E40" t="s">
-        <v>47</v>
-      </c>
-      <c r="F40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+      <c r="E42" t="s">
+        <v>47</v>
+      </c>
+      <c r="F42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>37</v>
       </c>
-      <c r="D41" s="6" t="s">
+      <c r="D43" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E41" t="s">
-        <v>47</v>
-      </c>
-      <c r="F41">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+      <c r="E43" t="s">
+        <v>47</v>
+      </c>
+      <c r="F43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>52</v>
       </c>
-      <c r="D42" s="6" t="s">
+      <c r="D44" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E42" t="s">
-        <v>47</v>
-      </c>
-      <c r="F42">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+      <c r="E44" t="s">
+        <v>47</v>
+      </c>
+      <c r="F44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>28</v>
       </c>
-      <c r="D43" s="6" t="s">
+      <c r="D45" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="E43" t="s">
-        <v>47</v>
-      </c>
-      <c r="F43">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+      <c r="E45" t="s">
+        <v>47</v>
+      </c>
+      <c r="F45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>10</v>
       </c>
-      <c r="D44" s="6" t="s">
+      <c r="D46" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="E44" t="s">
-        <v>47</v>
-      </c>
-      <c r="F44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+      <c r="E46" t="s">
+        <v>47</v>
+      </c>
+      <c r="F46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>62</v>
       </c>
-      <c r="D45" s="6" t="s">
+      <c r="D47" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="E45" t="s">
-        <v>47</v>
-      </c>
-      <c r="F45">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+      <c r="E47" t="s">
+        <v>47</v>
+      </c>
+      <c r="F47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>30</v>
       </c>
-      <c r="D46" s="6" t="s">
+      <c r="D48" s="6" t="s">
         <v>102</v>
-      </c>
-      <c r="E46" t="s">
-        <v>47</v>
-      </c>
-      <c r="F46">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>70</v>
-      </c>
-      <c r="D47" t="s">
-        <v>79</v>
-      </c>
-      <c r="E47" t="s">
-        <v>47</v>
-      </c>
-      <c r="F47">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>80</v>
-      </c>
-      <c r="D48" t="s">
-        <v>81</v>
       </c>
       <c r="E48" t="s">
         <v>47</v>
@@ -1738,206 +1771,200 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>70</v>
+      </c>
+      <c r="D49" t="s">
+        <v>79</v>
+      </c>
+      <c r="E49" t="s">
+        <v>47</v>
+      </c>
+      <c r="F49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>80</v>
+      </c>
+      <c r="D50" t="s">
+        <v>81</v>
+      </c>
+      <c r="E50" t="s">
+        <v>47</v>
+      </c>
+      <c r="F50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>55</v>
       </c>
-      <c r="D49" s="6" t="s">
+      <c r="D51" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="E49" t="s">
-        <v>47</v>
-      </c>
-      <c r="F49">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" s="4" t="s">
+      <c r="E51" t="s">
+        <v>47</v>
+      </c>
+      <c r="F51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D50" s="7" t="s">
+      <c r="D52" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="E50" t="s">
-        <v>47</v>
-      </c>
-      <c r="F50">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A51" s="4" t="s">
+      <c r="E52" t="s">
+        <v>47</v>
+      </c>
+      <c r="F52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B51" s="4"/>
-      <c r="D51" s="7" t="s">
+      <c r="B53" s="4"/>
+      <c r="D53" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="E51" t="s">
-        <v>47</v>
-      </c>
-      <c r="F51">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+      <c r="E53" t="s">
+        <v>47</v>
+      </c>
+      <c r="F53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>69</v>
       </c>
-      <c r="D52" s="6" t="s">
+      <c r="D54" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E52" t="s">
-        <v>47</v>
-      </c>
-      <c r="F52">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+      <c r="E54" t="s">
+        <v>47</v>
+      </c>
+      <c r="F54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
         <v>59</v>
       </c>
-      <c r="D53" s="6" t="s">
+      <c r="D55" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="E53" t="s">
-        <v>47</v>
-      </c>
-      <c r="F53">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A55" s="8" t="s">
+      <c r="E55" t="s">
+        <v>47</v>
+      </c>
+      <c r="F55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B55" s="8"/>
-      <c r="F55" s="4"/>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A56" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="E56" t="s">
-        <v>47</v>
-      </c>
-      <c r="F56" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A57" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B57" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="F57" s="9"/>
+      <c r="B57" s="8"/>
+      <c r="F57" s="4"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F58" s="9"/>
+        <v>156</v>
+      </c>
+      <c r="E58" t="s">
+        <v>47</v>
+      </c>
+      <c r="F58" s="9">
+        <v>0</v>
+      </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
-        <v>19</v>
+        <v>53</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="E59" t="s">
-        <v>47</v>
-      </c>
-      <c r="F59" s="9">
-        <v>0</v>
-      </c>
+        <v>158</v>
+      </c>
+      <c r="F59" s="9"/>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="F60" s="9"/>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A61" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="E61" t="s">
+        <v>47</v>
+      </c>
+      <c r="F61" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A62" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B60" s="4" t="s">
+      <c r="B62" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="E60" t="s">
-        <v>47</v>
-      </c>
-      <c r="F60" s="9">
+      <c r="E62" t="s">
+        <v>47</v>
+      </c>
+      <c r="F62" s="9">
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A61" s="4"/>
-      <c r="B61" s="4"/>
-      <c r="F61" s="4"/>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A62" s="1" t="s">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A63" s="4"/>
+      <c r="B63" s="4"/>
+      <c r="F63" s="4"/>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A64" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B62" s="1"/>
-      <c r="C62" s="1"/>
-      <c r="D62" s="1"/>
-      <c r="E62" s="1"/>
-      <c r="F62" s="1"/>
-      <c r="G62" s="12"/>
-      <c r="H62" s="1"/>
-      <c r="I62" s="1"/>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E63" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="F63" t="s">
-        <v>153</v>
-      </c>
-      <c r="G63" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="H63" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="I63" s="9" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E64" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="F64" t="s">
-        <v>153</v>
-      </c>
-      <c r="G64" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="H64" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="I64" s="9" t="s">
-        <v>161</v>
-      </c>
+      <c r="B64" s="1"/>
+      <c r="C64" s="1"/>
+      <c r="D64" s="1"/>
+      <c r="E64" s="1"/>
+      <c r="F64" s="1"/>
+      <c r="G64" s="12"/>
+      <c r="H64" s="1"/>
+      <c r="I64" s="1"/>
     </row>
     <row r="65" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E65" s="9" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="F65" t="s">
         <v>153</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H65" s="9" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="I65" s="9" t="s">
         <v>161</v>
@@ -1945,168 +1972,180 @@
     </row>
     <row r="66" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E66" s="9" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F66" t="s">
         <v>153</v>
       </c>
       <c r="G66" s="9" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="H66" s="9" t="s">
-        <v>144</v>
+        <v>151</v>
+      </c>
+      <c r="I66" s="9" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="67" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E67" s="9" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="F67" t="s">
         <v>153</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="H67" s="9" t="s">
-        <v>145</v>
+        <v>152</v>
+      </c>
+      <c r="I67" s="9" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="68" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E68" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F68" t="s">
         <v>153</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="69" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E69" s="9" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F69" t="s">
         <v>153</v>
       </c>
       <c r="G69" s="9" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H69" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="I69" s="9" t="s">
-        <v>164</v>
+        <v>145</v>
       </c>
     </row>
     <row r="70" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E70" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F70" t="s">
         <v>153</v>
       </c>
       <c r="G70" s="9" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="71" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E71" s="9" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F71" t="s">
         <v>153</v>
       </c>
       <c r="G71" s="9" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="H71" s="9" t="s">
-        <v>149</v>
+        <v>147</v>
+      </c>
+      <c r="I71" s="9" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="72" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E72" s="9" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F72" t="s">
         <v>153</v>
       </c>
       <c r="G72" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="H72" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="73" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E73" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="F73" t="s">
+        <v>153</v>
+      </c>
+      <c r="G73" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="H73" s="9" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="74" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E74" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="F74" t="s">
+        <v>153</v>
+      </c>
+      <c r="G74" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="H72" s="9" t="s">
+      <c r="H74" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="I72" s="9" t="s">
+      <c r="I74" s="9" t="s">
         <v>164</v>
-      </c>
-    </row>
-    <row r="73" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E73" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F73" s="5">
-        <v>0</v>
-      </c>
-      <c r="H73" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="74" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E74" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="F74" s="5">
-        <v>0</v>
-      </c>
-      <c r="G74" s="5"/>
-      <c r="H74" s="5" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="75" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E75" s="5" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="F75" s="5">
         <v>0</v>
       </c>
-      <c r="G75" s="5"/>
       <c r="H75" s="5" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="76" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E76" s="5" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F76" s="5">
         <v>0</v>
       </c>
+      <c r="G76" s="5"/>
       <c r="H76" s="5" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="77" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E77" s="5" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="F77" s="5">
         <v>0</v>
       </c>
+      <c r="G77" s="5"/>
       <c r="H77" s="5" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="78" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E78" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F78" s="5">
         <v>0</v>
@@ -2117,31 +2156,29 @@
     </row>
     <row r="79" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E79" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F79" s="5">
         <v>0</v>
       </c>
-      <c r="G79" s="5"/>
       <c r="H79" s="5" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="80" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E80" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F80" s="5">
         <v>0</v>
       </c>
-      <c r="G80" s="5"/>
       <c r="H80" s="5" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E81" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F81" s="5">
         <v>0</v>
@@ -2153,7 +2190,7 @@
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E82" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F82" s="5">
         <v>0</v>
@@ -2164,73 +2201,57 @@
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F83" s="4"/>
+      <c r="E83" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="F83" s="5">
+        <v>0</v>
+      </c>
+      <c r="G83" s="5"/>
+      <c r="H83" s="5" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A84" s="1" t="s">
+      <c r="E84" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="F84" s="5">
+        <v>0</v>
+      </c>
+      <c r="G84" s="5"/>
+      <c r="H84" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F85" s="4"/>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A86" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B84" s="1"/>
-      <c r="C84" s="1"/>
-      <c r="D84" s="1"/>
-      <c r="E84" s="2"/>
-      <c r="F84" s="2"/>
-      <c r="G84" s="2" t="s">
+      <c r="B86" s="1"/>
+      <c r="C86" s="1"/>
+      <c r="D86" s="1"/>
+      <c r="E86" s="2"/>
+      <c r="F86" s="2"/>
+      <c r="G86" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="H84" s="2"/>
-      <c r="I84" s="2"/>
-    </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E85" s="5" t="s">
+      <c r="H86" s="2"/>
+      <c r="I86" s="2"/>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E87" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="F85" s="5">
+      <c r="F87" s="5">
         <v>0</v>
       </c>
-      <c r="G85" s="5"/>
-      <c r="H85" s="5" t="s">
+      <c r="G87" s="5"/>
+      <c r="H87" s="5" t="s">
         <v>73</v>
-      </c>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>42</v>
-      </c>
-      <c r="C86" t="s">
-        <v>11</v>
-      </c>
-      <c r="D86" t="s">
-        <v>44</v>
-      </c>
-      <c r="E86" t="s">
-        <v>107</v>
-      </c>
-      <c r="F86">
-        <v>210</v>
-      </c>
-      <c r="I86" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>41</v>
-      </c>
-      <c r="C87" t="s">
-        <v>11</v>
-      </c>
-      <c r="D87" t="s">
-        <v>44</v>
-      </c>
-      <c r="E87" t="s">
-        <v>107</v>
-      </c>
-      <c r="F87" s="9">
-        <v>235</v>
-      </c>
-      <c r="I87" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -2238,7 +2259,7 @@
         <v>42</v>
       </c>
       <c r="C88" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D88" t="s">
         <v>44</v>
@@ -2246,11 +2267,11 @@
       <c r="E88" t="s">
         <v>107</v>
       </c>
-      <c r="F88" s="9">
-        <v>230</v>
+      <c r="F88">
+        <v>210</v>
       </c>
       <c r="I88" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -2258,7 +2279,7 @@
         <v>41</v>
       </c>
       <c r="C89" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D89" t="s">
         <v>44</v>
@@ -2267,61 +2288,64 @@
         <v>107</v>
       </c>
       <c r="F89" s="9">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="I89" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>34</v>
+        <v>42</v>
+      </c>
+      <c r="C90" t="s">
+        <v>12</v>
       </c>
       <c r="D90" t="s">
-        <v>75</v>
+        <v>44</v>
       </c>
       <c r="E90" t="s">
         <v>107</v>
       </c>
       <c r="F90" s="9">
-        <v>140</v>
+        <v>230</v>
       </c>
       <c r="I90" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>14</v>
+        <v>41</v>
+      </c>
+      <c r="C91" t="s">
+        <v>12</v>
       </c>
       <c r="D91" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="E91" t="s">
         <v>107</v>
       </c>
       <c r="F91" s="9">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="I91" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>13</v>
-      </c>
-      <c r="C92" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="D92" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E92" t="s">
         <v>107</v>
       </c>
       <c r="F92" s="9">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="I92" t="s">
         <v>108</v>
@@ -2331,9 +2355,6 @@
       <c r="A93" t="s">
         <v>14</v>
       </c>
-      <c r="C93" t="s">
-        <v>12</v>
-      </c>
       <c r="D93" t="s">
         <v>72</v>
       </c>
@@ -2341,10 +2362,10 @@
         <v>107</v>
       </c>
       <c r="F93" s="9">
-        <v>210</v>
-      </c>
-      <c r="H93" t="s">
-        <v>114</v>
+        <v>180</v>
+      </c>
+      <c r="I93" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -2352,7 +2373,7 @@
         <v>13</v>
       </c>
       <c r="C94" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D94" t="s">
         <v>72</v>
@@ -2361,47 +2382,47 @@
         <v>107</v>
       </c>
       <c r="F94" s="9">
-        <v>210</v>
+        <v>180</v>
       </c>
       <c r="I94" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="C95" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D95" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E95" t="s">
         <v>107</v>
       </c>
       <c r="F95" s="9">
-        <v>190</v>
-      </c>
-      <c r="I95" t="s">
-        <v>108</v>
+        <v>210</v>
+      </c>
+      <c r="H95" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="C96" t="s">
         <v>12</v>
       </c>
       <c r="D96" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E96" t="s">
         <v>107</v>
       </c>
       <c r="F96" s="9">
-        <v>230</v>
+        <v>210</v>
       </c>
       <c r="I96" t="s">
         <v>109</v>
@@ -2409,16 +2430,19 @@
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>40</v>
+        <v>27</v>
+      </c>
+      <c r="C97" t="s">
+        <v>11</v>
       </c>
       <c r="D97" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="E97" t="s">
         <v>107</v>
       </c>
-      <c r="F97">
-        <v>180</v>
+      <c r="F97" s="9">
+        <v>190</v>
       </c>
       <c r="I97" t="s">
         <v>108</v>
@@ -2426,527 +2450,558 @@
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>39</v>
+        <v>27</v>
+      </c>
+      <c r="C98" t="s">
+        <v>12</v>
       </c>
       <c r="D98" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="E98" t="s">
         <v>107</v>
       </c>
-      <c r="F98">
+      <c r="F98" s="9">
+        <v>230</v>
+      </c>
+      <c r="I98" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99" t="s">
+        <v>83</v>
+      </c>
+      <c r="E99" t="s">
+        <v>107</v>
+      </c>
+      <c r="F99">
         <v>180</v>
       </c>
-      <c r="H98" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A99" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B99" s="4"/>
+      <c r="I99" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A100" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B100" s="4"/>
-      <c r="D100" s="4" t="s">
-        <v>76</v>
+      <c r="A100" t="s">
+        <v>39</v>
+      </c>
+      <c r="D100" t="s">
+        <v>83</v>
       </c>
       <c r="E100" t="s">
         <v>107</v>
       </c>
-      <c r="F100" s="4">
-        <v>100</v>
+      <c r="F100">
+        <v>180</v>
+      </c>
+      <c r="H100" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B101" s="4"/>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A102" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B101" s="4"/>
-      <c r="D101" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E101" t="s">
-        <v>107</v>
-      </c>
-      <c r="F101" s="4">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>32</v>
-      </c>
-      <c r="C102" t="s">
-        <v>11</v>
-      </c>
-      <c r="D102" t="s">
-        <v>84</v>
+      <c r="B102" s="4"/>
+      <c r="D102" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="E102" t="s">
         <v>107</v>
       </c>
-      <c r="F102">
-        <v>20</v>
-      </c>
-      <c r="H102" t="s">
-        <v>111</v>
-      </c>
-      <c r="I102" t="s">
-        <v>108</v>
+      <c r="F102" s="4">
+        <v>100</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>32</v>
-      </c>
-      <c r="C103" t="s">
-        <v>12</v>
-      </c>
-      <c r="D103" t="s">
-        <v>84</v>
+      <c r="A103" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B103" s="4"/>
+      <c r="D103" s="4" t="s">
+        <v>75</v>
       </c>
       <c r="E103" t="s">
         <v>107</v>
       </c>
-      <c r="F103">
-        <v>21</v>
-      </c>
-      <c r="H103" t="s">
+      <c r="F103" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>32</v>
+      </c>
+      <c r="C104" t="s">
+        <v>11</v>
+      </c>
+      <c r="D104" t="s">
+        <v>84</v>
+      </c>
+      <c r="E104" t="s">
+        <v>107</v>
+      </c>
+      <c r="F104">
+        <v>20</v>
+      </c>
+      <c r="H104" t="s">
         <v>111</v>
       </c>
-      <c r="I103" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A104" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B104" s="4"/>
+      <c r="I104" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="C105" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D105" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E105" t="s">
         <v>107</v>
       </c>
       <c r="F105">
+        <v>21</v>
+      </c>
+      <c r="H105" t="s">
+        <v>111</v>
+      </c>
+      <c r="I105" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A106" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B106" s="4"/>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>15</v>
+      </c>
+      <c r="C107" t="s">
+        <v>11</v>
+      </c>
+      <c r="D107" t="s">
+        <v>85</v>
+      </c>
+      <c r="E107" t="s">
+        <v>107</v>
+      </c>
+      <c r="F107">
         <v>9</v>
       </c>
-      <c r="I105" t="s">
+      <c r="I107" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
-        <v>15</v>
-      </c>
-      <c r="C106" t="s">
-        <v>12</v>
-      </c>
-      <c r="D106" t="s">
-        <v>85</v>
-      </c>
-      <c r="E106" t="s">
-        <v>107</v>
-      </c>
-      <c r="F106">
-        <v>9.5</v>
-      </c>
-      <c r="I106" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A107" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B107" s="4"/>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>67</v>
+        <v>15</v>
       </c>
       <c r="C108" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D108" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="E108" t="s">
         <v>107</v>
       </c>
       <c r="F108">
+        <v>9.5</v>
+      </c>
+      <c r="I108" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A109" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B109" s="4"/>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>67</v>
+      </c>
+      <c r="C110" t="s">
+        <v>11</v>
+      </c>
+      <c r="D110" t="s">
+        <v>82</v>
+      </c>
+      <c r="E110" t="s">
+        <v>107</v>
+      </c>
+      <c r="F110">
         <v>0.33</v>
       </c>
-      <c r="I108" t="s">
+      <c r="I110" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
         <v>67</v>
       </c>
-      <c r="C109" t="s">
+      <c r="C111" t="s">
         <v>12</v>
       </c>
-      <c r="D109" t="s">
+      <c r="D111" t="s">
         <v>82</v>
       </c>
-      <c r="E109" t="s">
+      <c r="E111" t="s">
         <v>107</v>
       </c>
-      <c r="F109">
+      <c r="F111">
         <f>(5+0.4)/2</f>
         <v>2.7</v>
       </c>
-      <c r="H109" t="s">
+      <c r="H111" t="s">
         <v>110</v>
       </c>
-      <c r="I109" t="s">
+      <c r="I111" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
         <v>66</v>
       </c>
-      <c r="D110" t="s">
+      <c r="D112" t="s">
         <v>82</v>
       </c>
-      <c r="E110" t="s">
+      <c r="E112" t="s">
         <v>107</v>
       </c>
-      <c r="F110">
+      <c r="F112">
         <v>0.67</v>
       </c>
-      <c r="I110" t="s">
+      <c r="I112" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
         <v>64</v>
       </c>
-      <c r="D111" t="s">
+      <c r="D113" t="s">
         <v>78</v>
       </c>
-      <c r="E111" t="s">
+      <c r="E113" t="s">
         <v>107</v>
       </c>
-      <c r="F111">
+      <c r="F113">
         <f>900+1800</f>
         <v>2700</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
         <v>63</v>
       </c>
-      <c r="D112" t="s">
+      <c r="D114" t="s">
         <v>77</v>
-      </c>
-      <c r="E112" t="s">
-        <v>107</v>
-      </c>
-      <c r="F112">
-        <v>2000</v>
-      </c>
-      <c r="H112" t="s">
-        <v>112</v>
-      </c>
-      <c r="I112" s="10" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A113" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B113" s="4"/>
-      <c r="H113" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A114" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B114" s="4"/>
-      <c r="D114" t="s">
-        <v>95</v>
       </c>
       <c r="E114" t="s">
         <v>107</v>
       </c>
-      <c r="F114" s="4">
-        <v>5</v>
+      <c r="F114">
+        <v>2000</v>
+      </c>
+      <c r="H114" t="s">
+        <v>112</v>
+      </c>
+      <c r="I114" s="10" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" s="4" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="B115" s="4"/>
+      <c r="H115" s="4" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="B116" s="4"/>
+      <c r="D116" t="s">
+        <v>95</v>
+      </c>
+      <c r="E116" t="s">
+        <v>107</v>
+      </c>
+      <c r="F116" s="4">
+        <v>5</v>
+      </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" s="4" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="B117" s="4"/>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B118" s="4"/>
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A119" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B119" s="4"/>
+    </row>
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A120" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B118" s="4"/>
-    </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A119" s="9" t="s">
+      <c r="B120" s="4"/>
+    </row>
+    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A121" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B119" s="4"/>
-      <c r="D119" t="s">
+      <c r="B121" s="4"/>
+      <c r="D121" t="s">
         <v>95</v>
       </c>
-      <c r="E119" t="s">
+      <c r="E121" t="s">
         <v>107</v>
       </c>
-      <c r="F119">
+      <c r="F121">
         <v>7</v>
       </c>
-      <c r="H119" s="4" t="s">
+      <c r="H121" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="I119" t="s">
+      <c r="I121" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A120" s="9" t="s">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A122" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B120" s="4"/>
-      <c r="D120" t="s">
+      <c r="B122" s="4"/>
+      <c r="D122" t="s">
         <v>95</v>
       </c>
-      <c r="E120" t="s">
+      <c r="E122" t="s">
         <v>107</v>
       </c>
-      <c r="F120">
+      <c r="F122">
         <v>4</v>
       </c>
-      <c r="H120" s="4" t="s">
+      <c r="H122" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="I120" t="s">
+      <c r="I122" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A121" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B121" s="4"/>
-      <c r="H121" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A122" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B122" s="4"/>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" s="4" t="s">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="B123" s="4"/>
+      <c r="H123" s="4" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B124" s="4"/>
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A125" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B125" s="4"/>
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A126" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B124" s="4"/>
-    </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A125" s="9" t="s">
+      <c r="B126" s="4"/>
+    </row>
+    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A127" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B125" s="9"/>
-      <c r="C125" s="9"/>
-      <c r="D125" s="9"/>
-      <c r="E125" s="9"/>
-      <c r="F125" s="9">
+      <c r="B127" s="9"/>
+      <c r="C127" s="9"/>
+      <c r="D127" s="9"/>
+      <c r="E127" s="9"/>
+      <c r="F127" s="3">
         <v>0</v>
       </c>
-      <c r="H125" t="s">
+      <c r="H127" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A126" s="9" t="s">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A128" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B128" s="9"/>
+      <c r="C128" s="9"/>
+      <c r="D128" s="9"/>
+      <c r="E128" s="9"/>
+      <c r="F128" s="3">
+        <v>0</v>
+      </c>
+      <c r="H128" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A129" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B129" s="9"/>
+      <c r="C129" s="9"/>
+      <c r="D129" s="9"/>
+      <c r="E129" s="9"/>
+      <c r="F129" s="9">
+        <v>0</v>
+      </c>
+      <c r="H129" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A130" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B126" s="9"/>
-      <c r="C126" s="9"/>
-      <c r="D126" s="9"/>
-      <c r="E126" s="9"/>
-      <c r="F126" s="9">
+      <c r="B130" s="9"/>
+      <c r="C130" s="9"/>
+      <c r="D130" s="9"/>
+      <c r="E130" s="9"/>
+      <c r="F130" s="9">
         <v>0</v>
       </c>
-      <c r="H126" t="s">
+      <c r="H130" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A127" s="4" t="s">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A131" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B127" s="4"/>
-    </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A128" s="4" t="s">
+      <c r="B131" s="4"/>
+    </row>
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A132" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B128" s="4"/>
-    </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A129" s="4" t="s">
+      <c r="B132" s="4"/>
+    </row>
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A133" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B129" s="4"/>
-    </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A130" s="4" t="s">
+      <c r="B133" s="4"/>
+    </row>
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A134" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B130" s="4"/>
-    </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A131" s="4" t="s">
+      <c r="B134" s="4"/>
+    </row>
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A135" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B131" s="4"/>
-    </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A132" s="4" t="s">
+      <c r="B135" s="4"/>
+    </row>
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A136" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B132" s="4"/>
-    </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A133" s="4" t="s">
+      <c r="B136" s="4"/>
+    </row>
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A137" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B133" s="4"/>
-    </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A134" s="4" t="s">
+      <c r="B137" s="4"/>
+    </row>
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A138" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B134" s="4"/>
-    </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A135" s="4" t="s">
+      <c r="B138" s="4"/>
+    </row>
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A139" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B135" s="4"/>
-    </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A136" s="4" t="s">
+      <c r="B139" s="4"/>
+    </row>
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A140" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B136" s="4"/>
-    </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A137" s="4" t="s">
+      <c r="B140" s="4"/>
+    </row>
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A141" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B137" s="4"/>
-    </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A138" s="4" t="s">
+      <c r="B141" s="4"/>
+    </row>
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A142" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B138" s="4"/>
-    </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A139" s="4" t="s">
+      <c r="B142" s="4"/>
+    </row>
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A143" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B139" s="4"/>
-    </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A140" s="4" t="s">
+      <c r="B143" s="4"/>
+    </row>
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A144" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B140" s="4"/>
-    </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A141" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B141" s="4"/>
-    </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A142" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B142" s="4"/>
-      <c r="G142" s="4" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A143" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="B143" s="4"/>
-      <c r="G143" s="4" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A144" s="4" t="s">
-        <v>55</v>
-      </c>
       <c r="B144" s="4"/>
-      <c r="G144" s="4" t="s">
-        <v>166</v>
-      </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" s="4" t="s">
-        <v>61</v>
+        <v>30</v>
       </c>
       <c r="B145" s="4"/>
-      <c r="G145" s="4" t="s">
-        <v>166</v>
-      </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" s="4" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="B146" s="4"/>
       <c r="G146" s="4" t="s">
@@ -2955,7 +3010,7 @@
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" s="4" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="B147" s="4"/>
       <c r="G147" s="4" t="s">
@@ -2964,7 +3019,7 @@
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" s="4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B148" s="4"/>
       <c r="G148" s="4" t="s">
@@ -2972,739 +3027,833 @@
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F149" s="4"/>
+      <c r="A149" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B149" s="4"/>
+      <c r="G149" s="4" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A150" s="1" t="s">
+      <c r="A150" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B150" s="4"/>
+      <c r="G150" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A151" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B151" s="4"/>
+      <c r="G151" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A152" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B152" s="4"/>
+      <c r="G152" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F153" s="4"/>
+    </row>
+    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A154" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B150" s="1"/>
-      <c r="C150" s="1"/>
-      <c r="D150" s="1"/>
-      <c r="E150" s="2"/>
-      <c r="F150" s="2"/>
-      <c r="G150" s="2"/>
-      <c r="H150" s="2"/>
-      <c r="I150" s="2"/>
-    </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B151" t="s">
+      <c r="B154" s="1"/>
+      <c r="C154" s="1"/>
+      <c r="D154" s="1"/>
+      <c r="E154" s="2"/>
+      <c r="F154" s="2"/>
+      <c r="G154" s="2"/>
+      <c r="H154" s="2"/>
+      <c r="I154" s="2"/>
+    </row>
+    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B155" t="s">
         <v>49</v>
       </c>
-      <c r="E151" t="s">
+      <c r="E155" t="s">
         <v>122</v>
       </c>
-      <c r="F151" s="11">
+      <c r="F155" s="11">
         <f>1/7*100</f>
         <v>14.285714285714285</v>
       </c>
-      <c r="G151" t="s">
+      <c r="G155" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B152" t="s">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B156" t="s">
         <v>49</v>
       </c>
-      <c r="C152" t="s">
+      <c r="C156" t="s">
         <v>12</v>
       </c>
-      <c r="E152" t="s">
+      <c r="E156" t="s">
         <v>122</v>
       </c>
-      <c r="F152" s="4">
+      <c r="F156" s="4">
         <f>1/8*100</f>
         <v>12.5</v>
       </c>
-      <c r="G152" t="s">
+      <c r="G156" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B153" t="s">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B157" t="s">
         <v>48</v>
       </c>
-      <c r="E153" t="s">
+      <c r="E157" t="s">
         <v>122</v>
       </c>
-      <c r="F153" s="11">
+      <c r="F157" s="11">
         <f>1/6*100</f>
         <v>16.666666666666664</v>
       </c>
-      <c r="G153" t="s">
+      <c r="G157" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B154" t="s">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B158" t="s">
         <v>48</v>
       </c>
-      <c r="C154" t="s">
+      <c r="C158" t="s">
         <v>12</v>
       </c>
-      <c r="E154" t="s">
+      <c r="E158" t="s">
         <v>122</v>
       </c>
-      <c r="F154" s="11">
+      <c r="F158" s="11">
         <f>1/10*100</f>
         <v>10</v>
       </c>
-      <c r="G154" t="s">
+      <c r="G158" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F155" s="4"/>
-    </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A156" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="B156" s="1"/>
-      <c r="C156" s="1"/>
-      <c r="D156" s="1"/>
-      <c r="E156" s="2"/>
-      <c r="F156" s="2"/>
-      <c r="G156" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="H156" s="2"/>
-      <c r="I156" s="2"/>
-    </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E157" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F157" s="5">
-        <v>0</v>
-      </c>
-      <c r="G157" s="5"/>
-      <c r="H157" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E158" t="s">
-        <v>7</v>
-      </c>
-      <c r="F158" t="s">
-        <v>154</v>
-      </c>
-      <c r="H158" t="s">
-        <v>124</v>
-      </c>
-      <c r="I158" t="s">
-        <v>8</v>
-      </c>
+    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F159" s="4"/>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
-        <v>126</v>
+        <v>169</v>
       </c>
       <c r="B160" s="1"/>
       <c r="C160" s="1"/>
       <c r="D160" s="1"/>
       <c r="E160" s="2"/>
       <c r="F160" s="2"/>
-      <c r="G160" s="2"/>
+      <c r="G160" s="2" t="s">
+        <v>167</v>
+      </c>
       <c r="H160" s="2"/>
       <c r="I160" s="2"/>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A162" t="s">
+    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E161" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F161" s="5">
+        <v>0</v>
+      </c>
+      <c r="G161" s="5"/>
+      <c r="H161" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E162" t="s">
+        <v>7</v>
+      </c>
+      <c r="F162" t="s">
+        <v>154</v>
+      </c>
+      <c r="H162" t="s">
+        <v>124</v>
+      </c>
+      <c r="I162" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="164" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A164" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B164" s="1"/>
+      <c r="C164" s="1"/>
+      <c r="D164" s="1"/>
+      <c r="E164" s="2"/>
+      <c r="F164" s="2"/>
+      <c r="G164" s="2"/>
+      <c r="H164" s="2"/>
+      <c r="I164" s="2"/>
+    </row>
+    <row r="166" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
         <v>10</v>
       </c>
-      <c r="E162" t="s">
-        <v>125</v>
-      </c>
-      <c r="F162">
-        <v>1508</v>
-      </c>
-      <c r="G162" t="s">
+      <c r="E166" t="s">
+        <v>125</v>
+      </c>
+      <c r="F166">
+        <v>1507</v>
+      </c>
+      <c r="G166" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A163" t="s">
+    <row r="167" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
         <v>13</v>
       </c>
-      <c r="E163" t="s">
-        <v>125</v>
-      </c>
-      <c r="F163">
-        <v>980</v>
-      </c>
-    </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A164" t="s">
+      <c r="E167" t="s">
+        <v>125</v>
+      </c>
+      <c r="F167">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="168" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
         <v>14</v>
       </c>
-      <c r="E164" t="s">
-        <v>125</v>
-      </c>
-      <c r="F164">
-        <v>1212</v>
-      </c>
-    </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A165" t="s">
+      <c r="E168" t="s">
+        <v>125</v>
+      </c>
+      <c r="F168">
+        <v>1211</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
         <v>74</v>
       </c>
-      <c r="E165" t="s">
-        <v>125</v>
-      </c>
-      <c r="F165">
+      <c r="E169" t="s">
+        <v>125</v>
+      </c>
+      <c r="F169">
         <v>1779</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A166" t="s">
+    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
         <v>15</v>
       </c>
-      <c r="E166" t="s">
-        <v>125</v>
-      </c>
-      <c r="F166">
+      <c r="E170" t="s">
+        <v>125</v>
+      </c>
+      <c r="F170">
         <v>1092</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A167" t="s">
+    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
         <v>16</v>
       </c>
-      <c r="E167" t="s">
-        <v>125</v>
-      </c>
-      <c r="F167">
-        <v>1016</v>
-      </c>
-    </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A168" t="s">
+      <c r="E171" t="s">
+        <v>125</v>
+      </c>
+      <c r="F171">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
         <v>50</v>
       </c>
-      <c r="E168" t="s">
-        <v>125</v>
-      </c>
-      <c r="F168">
-        <v>1016</v>
-      </c>
-    </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A169" t="s">
+      <c r="E172" t="s">
+        <v>125</v>
+      </c>
+      <c r="F172">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
         <v>17</v>
       </c>
-      <c r="E169" t="s">
-        <v>125</v>
-      </c>
-      <c r="F169">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A170" t="s">
+      <c r="E173" t="s">
+        <v>125</v>
+      </c>
+      <c r="F173">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
         <v>51</v>
       </c>
-      <c r="E170" t="s">
-        <v>125</v>
-      </c>
-      <c r="F170">
+      <c r="E174" t="s">
+        <v>125</v>
+      </c>
+      <c r="F174">
         <v>1185</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A171" t="s">
+    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
         <v>80</v>
       </c>
-      <c r="E171" t="s">
-        <v>125</v>
-      </c>
-      <c r="F171">
-        <v>1016</v>
-      </c>
-    </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A172" t="s">
+      <c r="E175" t="s">
+        <v>125</v>
+      </c>
+      <c r="F175">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="176" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
         <v>52</v>
       </c>
-      <c r="E172" t="s">
-        <v>125</v>
-      </c>
-      <c r="F172">
-        <v>945</v>
-      </c>
-    </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A173" t="s">
-        <v>53</v>
-      </c>
-      <c r="E173" t="s">
-        <v>125</v>
-      </c>
-      <c r="F173">
-        <v>945</v>
-      </c>
-    </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A174" t="s">
-        <v>18</v>
-      </c>
-      <c r="E174" t="s">
-        <v>125</v>
-      </c>
-      <c r="F174">
-        <v>628</v>
-      </c>
-    </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A175" t="s">
-        <v>19</v>
-      </c>
-      <c r="E175" t="s">
-        <v>125</v>
-      </c>
-      <c r="F175">
-        <v>1016</v>
-      </c>
-    </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A176" t="s">
-        <v>20</v>
-      </c>
       <c r="E176" t="s">
         <v>125</v>
       </c>
       <c r="F176">
-        <v>1185</v>
+        <v>944</v>
       </c>
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E177" t="s">
         <v>125</v>
       </c>
       <c r="F177">
-        <v>1092</v>
+        <v>944</v>
       </c>
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E178" t="s">
         <v>125</v>
       </c>
       <c r="F178">
-        <v>1016</v>
+        <v>628</v>
       </c>
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="E179" t="s">
         <v>125</v>
       </c>
       <c r="F179">
-        <v>1475</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E180" t="s">
         <v>125</v>
       </c>
       <c r="F180">
-        <v>628</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="E181" t="s">
         <v>125</v>
       </c>
       <c r="F181">
-        <v>628</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E182" t="s">
         <v>125</v>
       </c>
       <c r="F182">
-        <v>1074</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E183" t="s">
         <v>125</v>
       </c>
       <c r="F183">
-        <v>628</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E184" t="s">
         <v>125</v>
       </c>
       <c r="F184">
-        <v>1487</v>
+        <v>628</v>
       </c>
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E185" t="s">
         <v>125</v>
       </c>
       <c r="F185">
-        <v>1487</v>
+        <v>628</v>
       </c>
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E186" t="s">
         <v>125</v>
       </c>
       <c r="F186">
-        <v>649</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="E187" t="s">
         <v>125</v>
       </c>
       <c r="F187">
-        <v>980</v>
+        <v>628</v>
       </c>
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="E188" t="s">
         <v>125</v>
       </c>
       <c r="F188">
-        <v>1074</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E189" t="s">
         <v>125</v>
       </c>
       <c r="F189">
-        <v>945</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E190" t="s">
         <v>125</v>
       </c>
       <c r="F190">
-        <v>1016</v>
+        <v>648</v>
       </c>
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E191" t="s">
         <v>125</v>
       </c>
       <c r="F191">
-        <v>767</v>
+        <v>979</v>
       </c>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="E192" t="s">
         <v>125</v>
       </c>
       <c r="F192">
-        <v>1508</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="E193" t="s">
         <v>125</v>
       </c>
       <c r="F193">
-        <v>1016</v>
+        <v>944</v>
       </c>
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="E194" t="s">
         <v>125</v>
       </c>
       <c r="F194">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="E195" t="s">
         <v>125</v>
       </c>
       <c r="F195">
-        <v>1185</v>
+        <v>766</v>
       </c>
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="E196" t="s">
         <v>125</v>
       </c>
       <c r="F196">
-        <v>1508</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="E197" t="s">
         <v>125</v>
       </c>
       <c r="F197">
-        <v>1212</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E198" t="s">
         <v>125</v>
       </c>
       <c r="F198">
-        <v>1569</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E199" t="s">
         <v>125</v>
       </c>
       <c r="F199">
-        <v>1569</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E200" t="s">
         <v>125</v>
       </c>
       <c r="F200">
-        <v>767</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="E201" t="s">
         <v>125</v>
       </c>
       <c r="F201">
-        <v>1185</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="E202" t="s">
         <v>125</v>
       </c>
       <c r="F202">
-        <v>1016</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E203" t="s">
         <v>125</v>
       </c>
       <c r="F203">
-        <v>1212</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="E204" t="s">
         <v>125</v>
       </c>
       <c r="F204">
-        <v>1016</v>
+        <v>766</v>
       </c>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="E205" t="s">
         <v>125</v>
       </c>
       <c r="F205">
-        <v>628</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="E206" t="s">
         <v>125</v>
       </c>
       <c r="F206">
-        <v>628</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E207" t="s">
         <v>125</v>
       </c>
       <c r="F207">
-        <v>1225</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
+        <v>34</v>
+      </c>
+      <c r="E208" t="s">
+        <v>125</v>
+      </c>
+      <c r="F208">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
+        <v>35</v>
+      </c>
+      <c r="E209" t="s">
+        <v>125</v>
+      </c>
+      <c r="F209">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
+        <v>36</v>
+      </c>
+      <c r="E210" t="s">
+        <v>125</v>
+      </c>
+      <c r="F210">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A211" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E211" t="s">
+        <v>125</v>
+      </c>
+      <c r="F211">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A212" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E212" t="s">
+        <v>125</v>
+      </c>
+      <c r="F212">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A213" t="s">
+        <v>68</v>
+      </c>
+      <c r="E213" t="s">
+        <v>125</v>
+      </c>
+      <c r="F213">
+        <v>1224</v>
+      </c>
+    </row>
+    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A214" t="s">
         <v>37</v>
       </c>
-      <c r="E208" t="s">
-        <v>125</v>
-      </c>
-      <c r="F208">
-        <v>1016</v>
-      </c>
-    </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A209" t="s">
+      <c r="E214" t="s">
+        <v>125</v>
+      </c>
+      <c r="F214">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A215" t="s">
         <v>69</v>
       </c>
-      <c r="E209" t="s">
-        <v>125</v>
-      </c>
-      <c r="F209">
-        <v>1016</v>
-      </c>
-    </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A210" t="s">
+      <c r="E215" t="s">
+        <v>125</v>
+      </c>
+      <c r="F215">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
         <v>38</v>
       </c>
-      <c r="E210" t="s">
-        <v>125</v>
-      </c>
-      <c r="F210">
+      <c r="E216" t="s">
+        <v>125</v>
+      </c>
+      <c r="F216">
         <v>1721</v>
       </c>
     </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A211" t="s">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
         <v>70</v>
       </c>
-      <c r="E211" t="s">
-        <v>125</v>
-      </c>
-      <c r="F211">
-        <v>1016</v>
-      </c>
-    </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A212" t="s">
+      <c r="E217" t="s">
+        <v>125</v>
+      </c>
+      <c r="F217">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A218" t="s">
         <v>39</v>
       </c>
-      <c r="E212" t="s">
-        <v>125</v>
-      </c>
-      <c r="F212">
+      <c r="E218" t="s">
+        <v>125</v>
+      </c>
+      <c r="F218">
+        <v>1211</v>
+      </c>
+    </row>
+    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
+        <v>40</v>
+      </c>
+      <c r="E219" t="s">
+        <v>125</v>
+      </c>
+      <c r="F219">
+        <v>1211</v>
+      </c>
+    </row>
+    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
+        <v>41</v>
+      </c>
+      <c r="E220" t="s">
+        <v>125</v>
+      </c>
+      <c r="F220">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
+        <v>42</v>
+      </c>
+      <c r="E221" t="s">
+        <v>125</v>
+      </c>
+      <c r="F221">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A222" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="B222" s="13"/>
+      <c r="C222" s="13"/>
+      <c r="D222" s="13"/>
+      <c r="E222" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="F222" s="13">
         <v>1212</v>
       </c>
-    </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A213" t="s">
-        <v>40</v>
-      </c>
-      <c r="E213" t="s">
-        <v>125</v>
-      </c>
-      <c r="F213">
+      <c r="G222" s="13"/>
+      <c r="H222" s="13" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A223" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="B223" s="13"/>
+      <c r="C223" s="13"/>
+      <c r="D223" s="13"/>
+      <c r="E223" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="F223" s="13">
         <v>1212</v>
       </c>
-    </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A214" t="s">
-        <v>41</v>
-      </c>
-      <c r="E214" t="s">
-        <v>125</v>
-      </c>
-      <c r="F214">
-        <v>980</v>
-      </c>
-    </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A215" t="s">
-        <v>42</v>
-      </c>
-      <c r="E215" t="s">
-        <v>125</v>
-      </c>
-      <c r="F215">
-        <v>1016</v>
+      <c r="G223" s="13"/>
+      <c r="H223" s="13" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -3713,7 +3862,7 @@
     <sortCondition ref="C14:C9129"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="I112" r:id="rId1"/>
+    <hyperlink ref="I114" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>

</xml_diff>

<commit_message>
Changed mixed cereals to oats/barley instead of oats/peas
</commit_message>
<xml_diff>
--- a/data/default/CropProduction.xlsx
+++ b/data/default/CropProduction.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="182">
   <si>
     <t>f_crop</t>
   </si>
@@ -587,6 +587,9 @@
   </si>
   <si>
     <t>https://www2.jordbruksverket.se/webdav/files/SJV/trycksaker/Pdf_ovrigt/p8_15-2.pdf</t>
+  </si>
+  <si>
+    <t>Antar 50-50</t>
   </si>
 </sst>
 </file>
@@ -1208,33 +1211,39 @@
       <c r="A13" t="s">
         <v>57</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="E13" t="s">
-        <v>47</v>
-      </c>
-      <c r="F13" s="4">
-        <v>0.2</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>160</v>
+      <c r="D13" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F13" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="I13" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>57</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="E14" t="s">
-        <v>47</v>
-      </c>
-      <c r="F14" s="4">
-        <v>0.8</v>
-      </c>
-      <c r="G14" s="4" t="s">
+      <c r="E14" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="G14" s="9" t="s">
         <v>159</v>
       </c>
     </row>
@@ -2520,33 +2529,38 @@
       <c r="B101" s="4"/>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A102" s="4" t="s">
+      <c r="A102" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B102" s="4"/>
-      <c r="D102" s="4" t="s">
+      <c r="B102" s="9"/>
+      <c r="C102" s="9"/>
+      <c r="D102" s="9" t="s">
         <v>76</v>
       </c>
       <c r="E102" t="s">
         <v>107</v>
       </c>
-      <c r="F102" s="4">
+      <c r="F102" s="9">
         <v>100</v>
       </c>
+      <c r="I102" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A103" s="4" t="s">
+      <c r="A103" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B103" s="4"/>
-      <c r="D103" s="4" t="s">
-        <v>75</v>
+      <c r="B103" s="9"/>
+      <c r="C103" s="9"/>
+      <c r="D103" s="9" t="s">
+        <v>72</v>
       </c>
       <c r="E103" t="s">
         <v>107</v>
       </c>
-      <c r="F103" s="4">
-        <v>100</v>
+      <c r="F103" s="9">
+        <v>110</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated data from latest run of CIBUSmod.data_curation
</commit_message>
<xml_diff>
--- a/data/default/CropProduction.xlsx
+++ b/data/default/CropProduction.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="202">
   <si>
     <t>f_crop</t>
   </si>
@@ -647,6 +647,9 @@
   </si>
   <si>
     <t>assumption on DM</t>
+  </si>
+  <si>
+    <t>Buckwheat</t>
   </si>
 </sst>
 </file>
@@ -1033,7 +1036,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I242"/>
+  <dimension ref="A1:I243"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="30.42578125" customWidth="1"/>
@@ -4260,6 +4263,20 @@
       <c r="G242" s="9"/>
       <c r="H242" s="9" t="s">
         <v>199</v>
+      </c>
+    </row>
+    <row r="243" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A243" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="E243" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="F243" s="9">
+        <v>1212</v>
+      </c>
+      <c r="H243" s="9" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added missing frac_renew factor in calculating crop residues
</commit_message>
<xml_diff>
--- a/data/default/CropProduction.xlsx
+++ b/data/default/CropProduction.xlsx
@@ -10,7 +10,7 @@
     <sheet name="default" sheetId="1" r:id="rId1"/>
     <sheet name="references" sheetId="5" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="204">
   <si>
     <t>f_crop</t>
   </si>
@@ -650,6 +650,12 @@
   </si>
   <si>
     <t>Buckwheat</t>
+  </si>
+  <si>
+    <t>frac_renew</t>
+  </si>
+  <si>
+    <t>Fraction of below ground residues renewed annually</t>
   </si>
 </sst>
 </file>
@@ -1036,7 +1042,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I243"/>
+  <dimension ref="A1:I245"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="30.42578125" customWidth="1"/>
@@ -2332,31 +2338,34 @@
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E82" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F82" s="5">
-        <v>0</v>
-      </c>
-      <c r="H82" s="5" t="s">
-        <v>73</v>
+      <c r="E82" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F82" t="s">
+        <v>153</v>
+      </c>
+      <c r="G82" s="9"/>
+      <c r="H82" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="I82" s="9" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E83" s="5" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="F83" s="5">
         <v>0</v>
       </c>
-      <c r="G83" s="5"/>
       <c r="H83" s="5" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E84" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F84" s="5">
         <v>0</v>
@@ -2368,18 +2377,19 @@
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E85" s="5" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F85" s="5">
         <v>0</v>
       </c>
+      <c r="G85" s="5"/>
       <c r="H85" s="5" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E86" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F86" s="5">
         <v>0</v>
@@ -2390,7 +2400,7 @@
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E87" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F87" s="5">
         <v>0</v>
@@ -2401,19 +2411,18 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E88" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F88" s="5">
         <v>0</v>
       </c>
-      <c r="G88" s="5"/>
       <c r="H88" s="5" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E89" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F89" s="5">
         <v>0</v>
@@ -2425,7 +2434,7 @@
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E90" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F90" s="5">
         <v>0</v>
@@ -2437,7 +2446,7 @@
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E91" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F91" s="5">
         <v>0</v>
@@ -2448,73 +2457,57 @@
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F92" s="4"/>
+      <c r="E92" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="F92" s="5">
+        <v>0</v>
+      </c>
+      <c r="G92" s="5"/>
+      <c r="H92" s="5" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A93" s="1" t="s">
+      <c r="E93" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="F93" s="5">
+        <v>1</v>
+      </c>
+      <c r="G93" s="5"/>
+      <c r="H93" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F94" s="4"/>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A95" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B93" s="1"/>
-      <c r="C93" s="1"/>
-      <c r="D93" s="1"/>
-      <c r="E93" s="2"/>
-      <c r="F93" s="2"/>
-      <c r="G93" s="2" t="s">
+      <c r="B95" s="1"/>
+      <c r="C95" s="1"/>
+      <c r="D95" s="1"/>
+      <c r="E95" s="2"/>
+      <c r="F95" s="2"/>
+      <c r="G95" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="H93" s="2"/>
-      <c r="I93" s="2"/>
-    </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E94" s="5" t="s">
+      <c r="H95" s="2"/>
+      <c r="I95" s="2"/>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E96" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="F94" s="5">
+      <c r="F96" s="5">
         <v>0</v>
       </c>
-      <c r="G94" s="5"/>
-      <c r="H94" s="5" t="s">
+      <c r="G96" s="5"/>
+      <c r="H96" s="5" t="s">
         <v>73</v>
-      </c>
-    </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>42</v>
-      </c>
-      <c r="C95" t="s">
-        <v>11</v>
-      </c>
-      <c r="D95" t="s">
-        <v>44</v>
-      </c>
-      <c r="E95" t="s">
-        <v>107</v>
-      </c>
-      <c r="F95">
-        <v>210</v>
-      </c>
-      <c r="I95" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>41</v>
-      </c>
-      <c r="C96" t="s">
-        <v>11</v>
-      </c>
-      <c r="D96" t="s">
-        <v>44</v>
-      </c>
-      <c r="E96" t="s">
-        <v>107</v>
-      </c>
-      <c r="F96" s="9">
-        <v>235</v>
-      </c>
-      <c r="I96" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -2522,7 +2515,7 @@
         <v>42</v>
       </c>
       <c r="C97" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D97" t="s">
         <v>44</v>
@@ -2530,11 +2523,11 @@
       <c r="E97" t="s">
         <v>107</v>
       </c>
-      <c r="F97" s="9">
-        <v>230</v>
+      <c r="F97">
+        <v>210</v>
       </c>
       <c r="I97" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -2542,7 +2535,7 @@
         <v>41</v>
       </c>
       <c r="C98" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D98" t="s">
         <v>44</v>
@@ -2551,61 +2544,64 @@
         <v>107</v>
       </c>
       <c r="F98" s="9">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="I98" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>34</v>
+        <v>42</v>
+      </c>
+      <c r="C99" t="s">
+        <v>12</v>
       </c>
       <c r="D99" t="s">
-        <v>75</v>
+        <v>44</v>
       </c>
       <c r="E99" t="s">
         <v>107</v>
       </c>
       <c r="F99" s="9">
-        <v>140</v>
+        <v>230</v>
       </c>
       <c r="I99" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>14</v>
+        <v>41</v>
+      </c>
+      <c r="C100" t="s">
+        <v>12</v>
       </c>
       <c r="D100" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="E100" t="s">
         <v>107</v>
       </c>
       <c r="F100" s="9">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="I100" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>13</v>
-      </c>
-      <c r="C101" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="D101" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E101" t="s">
         <v>107</v>
       </c>
       <c r="F101" s="9">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="I101" t="s">
         <v>108</v>
@@ -2615,9 +2611,6 @@
       <c r="A102" t="s">
         <v>14</v>
       </c>
-      <c r="C102" t="s">
-        <v>12</v>
-      </c>
       <c r="D102" t="s">
         <v>72</v>
       </c>
@@ -2625,10 +2618,10 @@
         <v>107</v>
       </c>
       <c r="F102" s="9">
-        <v>210</v>
-      </c>
-      <c r="H102" t="s">
-        <v>114</v>
+        <v>180</v>
+      </c>
+      <c r="I102" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -2636,7 +2629,7 @@
         <v>13</v>
       </c>
       <c r="C103" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D103" t="s">
         <v>72</v>
@@ -2645,47 +2638,47 @@
         <v>107</v>
       </c>
       <c r="F103" s="9">
-        <v>210</v>
+        <v>180</v>
       </c>
       <c r="I103" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="C104" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D104" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E104" t="s">
         <v>107</v>
       </c>
       <c r="F104" s="9">
-        <v>190</v>
-      </c>
-      <c r="I104" t="s">
-        <v>108</v>
+        <v>210</v>
+      </c>
+      <c r="H104" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="C105" t="s">
         <v>12</v>
       </c>
       <c r="D105" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E105" t="s">
         <v>107</v>
       </c>
       <c r="F105" s="9">
-        <v>230</v>
+        <v>210</v>
       </c>
       <c r="I105" t="s">
         <v>109</v>
@@ -2693,16 +2686,19 @@
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>40</v>
+        <v>27</v>
+      </c>
+      <c r="C106" t="s">
+        <v>11</v>
       </c>
       <c r="D106" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="E106" t="s">
         <v>107</v>
       </c>
-      <c r="F106">
-        <v>180</v>
+      <c r="F106" s="9">
+        <v>190</v>
       </c>
       <c r="I106" t="s">
         <v>108</v>
@@ -2710,207 +2706,220 @@
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>39</v>
+        <v>27</v>
+      </c>
+      <c r="C107" t="s">
+        <v>12</v>
       </c>
       <c r="D107" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="E107" t="s">
         <v>107</v>
       </c>
-      <c r="F107">
+      <c r="F107" s="9">
+        <v>230</v>
+      </c>
+      <c r="I107" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>40</v>
+      </c>
+      <c r="D108" t="s">
+        <v>83</v>
+      </c>
+      <c r="E108" t="s">
+        <v>107</v>
+      </c>
+      <c r="F108">
         <v>180</v>
       </c>
-      <c r="H107" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A108" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B108" s="4"/>
+      <c r="I108" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A109" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B109" s="9"/>
-      <c r="C109" s="9"/>
-      <c r="D109" s="9" t="s">
-        <v>76</v>
+      <c r="A109" t="s">
+        <v>39</v>
+      </c>
+      <c r="D109" t="s">
+        <v>83</v>
       </c>
       <c r="E109" t="s">
         <v>107</v>
       </c>
-      <c r="F109" s="9">
+      <c r="F109">
+        <v>180</v>
+      </c>
+      <c r="H109" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A110" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B110" s="4"/>
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A111" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B111" s="9"/>
+      <c r="C111" s="9"/>
+      <c r="D111" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E111" t="s">
+        <v>107</v>
+      </c>
+      <c r="F111" s="9">
         <v>100</v>
       </c>
-      <c r="I109" t="s">
+      <c r="I111" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A110" s="9" t="s">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A112" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B110" s="9"/>
-      <c r="C110" s="9"/>
-      <c r="D110" s="9" t="s">
+      <c r="B112" s="9"/>
+      <c r="C112" s="9"/>
+      <c r="D112" s="9" t="s">
         <v>72</v>
-      </c>
-      <c r="E110" t="s">
-        <v>107</v>
-      </c>
-      <c r="F110" s="9">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A111" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="B111" s="5"/>
-      <c r="C111" s="5"/>
-      <c r="D111" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="E111" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="F111" s="5">
-        <v>0</v>
-      </c>
-      <c r="G111" s="5"/>
-      <c r="H111" s="5" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
-        <v>32</v>
-      </c>
-      <c r="C112" t="s">
-        <v>11</v>
-      </c>
-      <c r="D112" t="s">
-        <v>84</v>
       </c>
       <c r="E112" t="s">
         <v>107</v>
       </c>
-      <c r="F112">
+      <c r="F112" s="9">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A113" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="B113" s="5"/>
+      <c r="C113" s="5"/>
+      <c r="D113" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E113" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="F113" s="5">
+        <v>0</v>
+      </c>
+      <c r="G113" s="5"/>
+      <c r="H113" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>32</v>
+      </c>
+      <c r="C114" t="s">
+        <v>11</v>
+      </c>
+      <c r="D114" t="s">
+        <v>84</v>
+      </c>
+      <c r="E114" t="s">
+        <v>107</v>
+      </c>
+      <c r="F114">
         <v>20</v>
       </c>
-      <c r="H112" t="s">
+      <c r="H114" t="s">
         <v>111</v>
       </c>
-      <c r="I112" t="s">
+      <c r="I114" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
-        <v>32</v>
-      </c>
-      <c r="C113" t="s">
-        <v>12</v>
-      </c>
-      <c r="D113" t="s">
-        <v>84</v>
-      </c>
-      <c r="E113" t="s">
-        <v>107</v>
-      </c>
-      <c r="F113">
-        <v>21</v>
-      </c>
-      <c r="H113" t="s">
-        <v>111</v>
-      </c>
-      <c r="I113" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A114" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B114" s="4"/>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="C115" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D115" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E115" t="s">
         <v>107</v>
       </c>
       <c r="F115">
+        <v>21</v>
+      </c>
+      <c r="H115" t="s">
+        <v>111</v>
+      </c>
+      <c r="I115" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A116" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B116" s="4"/>
+    </row>
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>15</v>
+      </c>
+      <c r="C117" t="s">
+        <v>11</v>
+      </c>
+      <c r="D117" t="s">
+        <v>85</v>
+      </c>
+      <c r="E117" t="s">
+        <v>107</v>
+      </c>
+      <c r="F117">
         <v>9</v>
       </c>
-      <c r="I115" t="s">
+      <c r="I117" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
         <v>15</v>
       </c>
-      <c r="C116" t="s">
+      <c r="C118" t="s">
         <v>12</v>
       </c>
-      <c r="D116" t="s">
+      <c r="D118" t="s">
         <v>85</v>
       </c>
-      <c r="E116" t="s">
+      <c r="E118" t="s">
         <v>107</v>
       </c>
-      <c r="F116">
+      <c r="F118">
         <v>9.5</v>
       </c>
-      <c r="I116" t="s">
+      <c r="I118" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A117" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B117" s="4"/>
-    </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A118" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="B118" s="5"/>
-      <c r="C118" s="5"/>
-      <c r="D118" s="5"/>
-      <c r="E118" s="5"/>
-      <c r="F118" s="5"/>
-      <c r="G118" s="5"/>
-      <c r="H118" s="5"/>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="B119" s="5"/>
-      <c r="C119" s="5"/>
-      <c r="D119" s="5"/>
-      <c r="E119" s="5"/>
-      <c r="F119" s="5"/>
-      <c r="G119" s="5"/>
-      <c r="H119" s="5"/>
+        <v>74</v>
+      </c>
+      <c r="B119" s="4"/>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="B120" s="5"/>
       <c r="C120" s="5"/>
@@ -2921,89 +2930,93 @@
       <c r="H120" s="5"/>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
+      <c r="A121" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B121" s="5"/>
+      <c r="C121" s="5"/>
+      <c r="D121" s="5"/>
+      <c r="E121" s="5"/>
+      <c r="F121" s="5"/>
+      <c r="G121" s="5"/>
+      <c r="H121" s="5"/>
+    </row>
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A122" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B122" s="5"/>
+      <c r="C122" s="5"/>
+      <c r="D122" s="5"/>
+      <c r="E122" s="5"/>
+      <c r="F122" s="5"/>
+      <c r="G122" s="5"/>
+      <c r="H122" s="5"/>
+    </row>
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
         <v>67</v>
       </c>
-      <c r="C121" t="s">
+      <c r="C123" t="s">
         <v>11</v>
       </c>
-      <c r="D121" t="s">
+      <c r="D123" t="s">
         <v>82</v>
       </c>
-      <c r="E121" t="s">
+      <c r="E123" t="s">
         <v>107</v>
       </c>
-      <c r="F121">
+      <c r="F123">
         <v>0.33</v>
       </c>
-      <c r="I121" t="s">
+      <c r="I123" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
         <v>67</v>
       </c>
-      <c r="C122" t="s">
+      <c r="C124" t="s">
         <v>12</v>
       </c>
-      <c r="D122" t="s">
+      <c r="D124" t="s">
         <v>82</v>
       </c>
-      <c r="E122" t="s">
+      <c r="E124" t="s">
         <v>107</v>
       </c>
-      <c r="F122">
+      <c r="F124">
         <f>(5+0.4)/2</f>
         <v>2.7</v>
       </c>
-      <c r="H122" t="s">
+      <c r="H124" t="s">
         <v>110</v>
       </c>
-      <c r="I122" t="s">
+      <c r="I124" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
         <v>66</v>
       </c>
-      <c r="D123" t="s">
+      <c r="D125" t="s">
         <v>82</v>
       </c>
-      <c r="E123" t="s">
+      <c r="E125" t="s">
         <v>107</v>
       </c>
-      <c r="F123">
+      <c r="F125">
         <v>0.67</v>
       </c>
-      <c r="I123" t="s">
+      <c r="I125" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A124" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="B124" s="5"/>
-      <c r="C124" s="5"/>
-      <c r="D124" s="5"/>
-      <c r="E124" s="5"/>
-      <c r="F124" s="5"/>
-    </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A125" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="B125" s="5"/>
-      <c r="C125" s="5"/>
-      <c r="D125" s="5"/>
-      <c r="E125" s="5"/>
-      <c r="F125" s="5"/>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B126" s="5"/>
       <c r="C126" s="5"/>
@@ -3012,196 +3025,186 @@
       <c r="F126" s="5"/>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
+      <c r="A127" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B127" s="5"/>
+      <c r="C127" s="5"/>
+      <c r="D127" s="5"/>
+      <c r="E127" s="5"/>
+      <c r="F127" s="5"/>
+    </row>
+    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A128" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B128" s="5"/>
+      <c r="C128" s="5"/>
+      <c r="D128" s="5"/>
+      <c r="E128" s="5"/>
+      <c r="F128" s="5"/>
+    </row>
+    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
         <v>64</v>
       </c>
-      <c r="D127" t="s">
+      <c r="D129" t="s">
         <v>78</v>
       </c>
-      <c r="E127" t="s">
+      <c r="E129" t="s">
         <v>107</v>
       </c>
-      <c r="F127">
+      <c r="F129">
         <f>900+1800</f>
         <v>2700</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
         <v>63</v>
       </c>
-      <c r="D128" t="s">
+      <c r="D130" t="s">
         <v>77</v>
-      </c>
-      <c r="E128" t="s">
-        <v>107</v>
-      </c>
-      <c r="F128">
-        <v>2000</v>
-      </c>
-      <c r="H128" t="s">
-        <v>112</v>
-      </c>
-      <c r="I128" s="10" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A129" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B129" s="4"/>
-      <c r="H129" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A130" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B130" s="4"/>
-      <c r="D130" t="s">
-        <v>95</v>
       </c>
       <c r="E130" t="s">
         <v>107</v>
       </c>
-      <c r="F130" s="4">
-        <v>5</v>
+      <c r="F130">
+        <v>2000</v>
+      </c>
+      <c r="H130" t="s">
+        <v>112</v>
+      </c>
+      <c r="I130" s="10" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" s="4" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="B131" s="4"/>
+      <c r="H131" s="4" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="B132" s="4"/>
+      <c r="D132" t="s">
+        <v>95</v>
+      </c>
+      <c r="E132" t="s">
+        <v>107</v>
+      </c>
+      <c r="F132" s="4">
+        <v>5</v>
+      </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" s="4" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="B133" s="4"/>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B134" s="4"/>
+    </row>
+    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A135" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B135" s="4"/>
+    </row>
+    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A136" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B134" s="4"/>
-    </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A135" s="9" t="s">
+      <c r="B136" s="4"/>
+    </row>
+    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A137" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B135" s="4"/>
-      <c r="D135" t="s">
+      <c r="B137" s="4"/>
+      <c r="D137" t="s">
         <v>95</v>
       </c>
-      <c r="E135" t="s">
+      <c r="E137" t="s">
         <v>107</v>
       </c>
-      <c r="F135">
+      <c r="F137">
         <v>7</v>
       </c>
-      <c r="H135" s="4" t="s">
+      <c r="H137" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="I135" t="s">
+      <c r="I137" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A136" s="9" t="s">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A138" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B136" s="4"/>
-      <c r="D136" t="s">
+      <c r="B138" s="4"/>
+      <c r="D138" t="s">
         <v>95</v>
       </c>
-      <c r="E136" t="s">
+      <c r="E138" t="s">
         <v>107</v>
       </c>
-      <c r="F136">
+      <c r="F138">
         <v>4</v>
       </c>
-      <c r="H136" s="4" t="s">
+      <c r="H138" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="I136" t="s">
+      <c r="I138" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A137" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B137" s="4"/>
-      <c r="H137" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A138" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B138" s="4"/>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" s="4" t="s">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="B139" s="4"/>
+      <c r="H139" s="4" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B140" s="4"/>
+    </row>
+    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A141" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B141" s="4"/>
+    </row>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A142" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B140" s="4"/>
-    </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A141" s="9" t="s">
+      <c r="B142" s="4"/>
+    </row>
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A143" s="9" t="s">
         <v>36</v>
-      </c>
-      <c r="B141" s="9"/>
-      <c r="C141" s="9"/>
-      <c r="D141" s="9"/>
-      <c r="E141" s="9"/>
-      <c r="F141" s="3">
-        <v>0</v>
-      </c>
-      <c r="H141" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A142" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="B142" s="9"/>
-      <c r="C142" s="9"/>
-      <c r="D142" s="9"/>
-      <c r="E142" s="9"/>
-      <c r="F142" s="3">
-        <v>0</v>
-      </c>
-      <c r="H142" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A143" s="3" t="s">
-        <v>174</v>
       </c>
       <c r="B143" s="9"/>
       <c r="C143" s="9"/>
       <c r="D143" s="9"/>
       <c r="E143" s="9"/>
-      <c r="F143" s="9">
+      <c r="F143" s="3">
         <v>0</v>
       </c>
       <c r="H143" t="s">
@@ -3209,131 +3212,143 @@
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A144" s="9" t="s">
-        <v>35</v>
+      <c r="A144" s="3" t="s">
+        <v>173</v>
       </c>
       <c r="B144" s="9"/>
       <c r="C144" s="9"/>
       <c r="D144" s="9"/>
       <c r="E144" s="9"/>
-      <c r="F144" s="9">
+      <c r="F144" s="3">
         <v>0</v>
       </c>
       <c r="H144" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A145" s="4" t="s">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A145" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B145" s="9"/>
+      <c r="C145" s="9"/>
+      <c r="D145" s="9"/>
+      <c r="E145" s="9"/>
+      <c r="F145" s="9">
+        <v>0</v>
+      </c>
+      <c r="H145" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A146" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B146" s="9"/>
+      <c r="C146" s="9"/>
+      <c r="D146" s="9"/>
+      <c r="E146" s="9"/>
+      <c r="F146" s="9">
+        <v>0</v>
+      </c>
+      <c r="H146" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A147" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B145" s="4"/>
-    </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A146" s="4" t="s">
+      <c r="B147" s="4"/>
+    </row>
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A148" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B146" s="4"/>
-    </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A147" s="4" t="s">
+      <c r="B148" s="4"/>
+    </row>
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A149" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B147" s="4"/>
-    </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A148" s="4" t="s">
+      <c r="B149" s="4"/>
+    </row>
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A150" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B148" s="4"/>
-    </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A149" s="4" t="s">
+      <c r="B150" s="4"/>
+    </row>
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A151" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B149" s="4"/>
-    </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A150" s="4" t="s">
+      <c r="B151" s="4"/>
+    </row>
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A152" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B150" s="4"/>
-    </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A151" s="4" t="s">
+      <c r="B152" s="4"/>
+    </row>
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A153" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B151" s="4"/>
-    </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A152" s="4" t="s">
+      <c r="B153" s="4"/>
+    </row>
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A154" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B152" s="4"/>
-    </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A153" s="4" t="s">
+      <c r="B154" s="4"/>
+    </row>
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A155" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B153" s="4"/>
-    </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A154" s="4" t="s">
+      <c r="B155" s="4"/>
+    </row>
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A156" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B154" s="4"/>
-    </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A155" s="4" t="s">
+      <c r="B156" s="4"/>
+    </row>
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A157" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B155" s="4"/>
-    </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A156" s="4" t="s">
+      <c r="B157" s="4"/>
+    </row>
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A158" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B156" s="4"/>
-    </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A157" s="4" t="s">
+      <c r="B158" s="4"/>
+    </row>
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A159" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B157" s="4"/>
-    </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A158" s="4" t="s">
+      <c r="B159" s="4"/>
+    </row>
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A160" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B158" s="4"/>
-    </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A159" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B159" s="4"/>
-    </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A160" s="4" t="s">
-        <v>70</v>
-      </c>
       <c r="B160" s="4"/>
-      <c r="G160" s="4" t="s">
-        <v>166</v>
-      </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" s="4" t="s">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="B161" s="4"/>
-      <c r="G161" s="4" t="s">
-        <v>166</v>
-      </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" s="4" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="B162" s="4"/>
       <c r="G162" s="4" t="s">
@@ -3342,7 +3357,7 @@
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A163" s="4" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="B163" s="4"/>
       <c r="G163" s="4" t="s">
@@ -3351,7 +3366,7 @@
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B164" s="4"/>
       <c r="G164" s="4" t="s">
@@ -3360,7 +3375,7 @@
     </row>
     <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A165" s="4" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="B165" s="4"/>
       <c r="G165" s="4" t="s">
@@ -3369,7 +3384,7 @@
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A166" s="4" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B166" s="4"/>
       <c r="G166" s="4" t="s">
@@ -3377,384 +3392,380 @@
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F167" s="4"/>
+      <c r="A167" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B167" s="4"/>
+      <c r="G167" s="4" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A168" s="1" t="s">
+      <c r="A168" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B168" s="4"/>
+      <c r="G168" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F169" s="4"/>
+    </row>
+    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A170" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B168" s="1"/>
-      <c r="C168" s="1"/>
-      <c r="D168" s="1"/>
-      <c r="E168" s="2"/>
-      <c r="F168" s="2"/>
-      <c r="G168" s="2"/>
-      <c r="H168" s="2"/>
-      <c r="I168" s="2"/>
-    </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B169" t="s">
+      <c r="B170" s="1"/>
+      <c r="C170" s="1"/>
+      <c r="D170" s="1"/>
+      <c r="E170" s="2"/>
+      <c r="F170" s="2"/>
+      <c r="G170" s="2"/>
+      <c r="H170" s="2"/>
+      <c r="I170" s="2"/>
+    </row>
+    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B171" t="s">
         <v>49</v>
       </c>
-      <c r="E169" t="s">
+      <c r="E171" t="s">
         <v>122</v>
       </c>
-      <c r="F169" s="11">
+      <c r="F171" s="11">
         <f>1/7*100</f>
         <v>14.285714285714285</v>
       </c>
-      <c r="G169" t="s">
+      <c r="G171" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B170" t="s">
+    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B172" t="s">
         <v>49</v>
       </c>
-      <c r="C170" t="s">
+      <c r="C172" t="s">
         <v>12</v>
       </c>
-      <c r="E170" t="s">
+      <c r="E172" t="s">
         <v>122</v>
       </c>
-      <c r="F170" s="4">
+      <c r="F172" s="4">
         <f>1/8*100</f>
         <v>12.5</v>
       </c>
-      <c r="G170" t="s">
+      <c r="G172" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B171" t="s">
+    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B173" t="s">
         <v>48</v>
       </c>
-      <c r="E171" t="s">
+      <c r="E173" t="s">
         <v>122</v>
       </c>
-      <c r="F171" s="11">
+      <c r="F173" s="11">
         <f>1/6*100</f>
         <v>16.666666666666664</v>
       </c>
-      <c r="G171" t="s">
+      <c r="G173" t="s">
         <v>123</v>
       </c>
-      <c r="I171" t="s">
+      <c r="I173" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B172" t="s">
+    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B174" t="s">
         <v>48</v>
       </c>
-      <c r="C172" t="s">
+      <c r="C174" t="s">
         <v>12</v>
       </c>
-      <c r="E172" t="s">
+      <c r="E174" t="s">
         <v>122</v>
       </c>
-      <c r="F172" s="11">
+      <c r="F174" s="11">
         <f>1/10*100</f>
         <v>10</v>
       </c>
-      <c r="G172" t="s">
+      <c r="G174" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F173" s="4"/>
-    </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A174" s="1" t="s">
+    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F175" s="4"/>
+    </row>
+    <row r="176" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A176" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="B174" s="1"/>
-      <c r="C174" s="1"/>
-      <c r="D174" s="1"/>
-      <c r="E174" s="2"/>
-      <c r="F174" s="2"/>
-      <c r="G174" s="2" t="s">
+      <c r="B176" s="1"/>
+      <c r="C176" s="1"/>
+      <c r="D176" s="1"/>
+      <c r="E176" s="2"/>
+      <c r="F176" s="2"/>
+      <c r="G176" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="H174" s="2"/>
-      <c r="I174" s="2"/>
-    </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E175" s="5" t="s">
+      <c r="H176" s="2"/>
+      <c r="I176" s="2"/>
+    </row>
+    <row r="177" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E177" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F175" s="5">
+      <c r="F177" s="5">
         <v>0</v>
       </c>
-      <c r="G175" s="5"/>
-      <c r="H175" s="5" t="s">
+      <c r="G177" s="5"/>
+      <c r="H177" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E176" t="s">
+    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E178" t="s">
         <v>7</v>
       </c>
-      <c r="F176" t="s">
+      <c r="F178" t="s">
         <v>154</v>
       </c>
-      <c r="H176" t="s">
+      <c r="H178" t="s">
         <v>124</v>
       </c>
-      <c r="I176" t="s">
+      <c r="I178" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A178" s="1" t="s">
+    <row r="180" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A180" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B178" s="1"/>
-      <c r="C178" s="1"/>
-      <c r="D178" s="1"/>
-      <c r="E178" s="2"/>
-      <c r="F178" s="2"/>
-      <c r="G178" s="2"/>
-      <c r="H178" s="2"/>
-      <c r="I178" s="2"/>
-    </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A180" t="s">
-        <v>10</v>
-      </c>
-      <c r="E180" t="s">
-        <v>125</v>
-      </c>
-      <c r="F180">
-        <v>1507</v>
-      </c>
-      <c r="G180" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="181" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A181" t="s">
-        <v>13</v>
-      </c>
-      <c r="E181" t="s">
-        <v>125</v>
-      </c>
-      <c r="F181">
-        <v>979</v>
-      </c>
+      <c r="B180" s="1"/>
+      <c r="C180" s="1"/>
+      <c r="D180" s="1"/>
+      <c r="E180" s="2"/>
+      <c r="F180" s="2"/>
+      <c r="G180" s="2"/>
+      <c r="H180" s="2"/>
+      <c r="I180" s="2"/>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E182" t="s">
         <v>125</v>
       </c>
       <c r="F182">
-        <v>1211</v>
+        <v>1507</v>
+      </c>
+      <c r="G182" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="E183" t="s">
         <v>125</v>
       </c>
       <c r="F183">
-        <v>1779</v>
+        <v>979</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E184" t="s">
         <v>125</v>
       </c>
       <c r="F184">
-        <v>1092</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>16</v>
+        <v>74</v>
       </c>
       <c r="E185" t="s">
         <v>125</v>
       </c>
       <c r="F185">
-        <v>1015</v>
+        <v>1779</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="E186" t="s">
         <v>125</v>
       </c>
       <c r="F186">
-        <v>1015</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E187" t="s">
         <v>125</v>
       </c>
       <c r="F187">
-        <v>648</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="188" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E188" t="s">
         <v>125</v>
       </c>
       <c r="F188">
-        <v>1185</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>80</v>
+        <v>17</v>
       </c>
       <c r="E189" t="s">
         <v>125</v>
       </c>
       <c r="F189">
-        <v>1015</v>
+        <v>648</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E190" t="s">
         <v>125</v>
       </c>
       <c r="F190">
-        <v>944</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>53</v>
+        <v>80</v>
       </c>
       <c r="E191" t="s">
         <v>125</v>
       </c>
       <c r="F191">
-        <v>944</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="192" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="E192" t="s">
         <v>125</v>
       </c>
       <c r="F192">
-        <v>628</v>
+        <v>944</v>
       </c>
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>19</v>
+        <v>53</v>
       </c>
       <c r="E193" t="s">
         <v>125</v>
       </c>
       <c r="F193">
-        <v>1015</v>
+        <v>944</v>
       </c>
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E194" t="s">
         <v>125</v>
       </c>
       <c r="F194">
-        <v>1185</v>
+        <v>628</v>
       </c>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
       <c r="E195" t="s">
         <v>125</v>
       </c>
       <c r="F195">
-        <v>1092</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E196" t="s">
         <v>125</v>
       </c>
       <c r="F196">
-        <v>1015</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E197" t="s">
         <v>125</v>
       </c>
       <c r="F197">
-        <v>1474</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E198" t="s">
         <v>125</v>
       </c>
       <c r="F198">
-        <v>628</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="E199" t="s">
         <v>125</v>
       </c>
       <c r="F199">
-        <v>628</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E200" t="s">
         <v>125</v>
       </c>
       <c r="F200">
-        <v>1073</v>
+        <v>628</v>
       </c>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="E201" t="s">
         <v>125</v>
@@ -3765,227 +3776,227 @@
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E202" t="s">
         <v>125</v>
       </c>
       <c r="F202">
-        <v>1486</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="E203" t="s">
         <v>125</v>
       </c>
       <c r="F203">
-        <v>1486</v>
+        <v>628</v>
       </c>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="E204" t="s">
         <v>125</v>
       </c>
       <c r="F204">
-        <v>648</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E205" t="s">
         <v>125</v>
       </c>
       <c r="F205">
-        <v>979</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E206" t="s">
         <v>125</v>
       </c>
       <c r="F206">
-        <v>1073</v>
+        <v>648</v>
       </c>
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E207" t="s">
         <v>125</v>
       </c>
       <c r="F207">
-        <v>944</v>
+        <v>979</v>
       </c>
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E208" t="s">
         <v>125</v>
       </c>
       <c r="F208">
-        <v>1015</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E209" t="s">
         <v>125</v>
       </c>
       <c r="F209">
-        <v>766</v>
+        <v>944</v>
       </c>
     </row>
     <row r="210" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="E210" t="s">
         <v>125</v>
       </c>
       <c r="F210">
-        <v>1507</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="E211" t="s">
         <v>125</v>
       </c>
       <c r="F211">
-        <v>1015</v>
+        <v>766</v>
       </c>
     </row>
     <row r="212" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E212" t="s">
         <v>125</v>
       </c>
       <c r="F212">
-        <v>1015</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="213" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E213" t="s">
         <v>125</v>
       </c>
       <c r="F213">
-        <v>1185</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="214" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="E214" t="s">
         <v>125</v>
       </c>
       <c r="F214">
-        <v>1507</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="215" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="E215" t="s">
         <v>125</v>
       </c>
       <c r="F215">
-        <v>1211</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="216" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="E216" t="s">
         <v>125</v>
       </c>
       <c r="F216">
-        <v>1569</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="217" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="E217" t="s">
         <v>125</v>
       </c>
       <c r="F217">
-        <v>1569</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="218" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="E218" t="s">
         <v>125</v>
       </c>
       <c r="F218">
-        <v>766</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E219" t="s">
         <v>125</v>
       </c>
       <c r="F219">
-        <v>1185</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="220" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E220" t="s">
         <v>125</v>
       </c>
       <c r="F220">
-        <v>1015</v>
+        <v>766</v>
       </c>
     </row>
     <row r="221" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E221" t="s">
         <v>125</v>
       </c>
       <c r="F221">
-        <v>1211</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="222" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>34</v>
+        <v>66</v>
       </c>
       <c r="E222" t="s">
         <v>125</v>
@@ -3996,29 +4007,29 @@
     </row>
     <row r="223" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>35</v>
+        <v>67</v>
       </c>
       <c r="E223" t="s">
         <v>125</v>
       </c>
       <c r="F223">
-        <v>628</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="224" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E224" t="s">
         <v>125</v>
       </c>
       <c r="F224">
-        <v>628</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A225" s="3" t="s">
-        <v>173</v>
+      <c r="A225" t="s">
+        <v>35</v>
       </c>
       <c r="E225" t="s">
         <v>125</v>
@@ -4028,8 +4039,8 @@
       </c>
     </row>
     <row r="226" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A226" s="3" t="s">
-        <v>174</v>
+      <c r="A226" t="s">
+        <v>36</v>
       </c>
       <c r="E226" t="s">
         <v>125</v>
@@ -4039,52 +4050,52 @@
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A227" t="s">
-        <v>68</v>
+      <c r="A227" s="3" t="s">
+        <v>173</v>
       </c>
       <c r="E227" t="s">
         <v>125</v>
       </c>
       <c r="F227">
-        <v>1224</v>
+        <v>628</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A228" t="s">
-        <v>37</v>
+      <c r="A228" s="3" t="s">
+        <v>174</v>
       </c>
       <c r="E228" t="s">
         <v>125</v>
       </c>
       <c r="F228">
-        <v>1015</v>
+        <v>628</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E229" t="s">
         <v>125</v>
       </c>
       <c r="F229">
-        <v>1015</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E230" t="s">
         <v>125</v>
       </c>
       <c r="F230">
-        <v>1721</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E231" t="s">
         <v>125</v>
@@ -4095,89 +4106,73 @@
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E232" t="s">
         <v>125</v>
       </c>
       <c r="F232">
-        <v>1211</v>
+        <v>1721</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="E233" t="s">
         <v>125</v>
       </c>
       <c r="F233">
-        <v>1211</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E234" t="s">
         <v>125</v>
       </c>
       <c r="F234">
-        <v>979</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
+        <v>40</v>
+      </c>
+      <c r="E235" t="s">
+        <v>125</v>
+      </c>
+      <c r="F235">
+        <v>1211</v>
+      </c>
+    </row>
+    <row r="236" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A236" t="s">
+        <v>41</v>
+      </c>
+      <c r="E236" t="s">
+        <v>125</v>
+      </c>
+      <c r="F236">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="237" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A237" t="s">
         <v>42</v>
       </c>
-      <c r="E235" t="s">
-        <v>125</v>
-      </c>
-      <c r="F235">
+      <c r="E237" t="s">
+        <v>125</v>
+      </c>
+      <c r="F237">
         <v>1015</v>
       </c>
-    </row>
-    <row r="236" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A236" s="9" t="s">
-        <v>175</v>
-      </c>
-      <c r="B236" s="9"/>
-      <c r="C236" s="9"/>
-      <c r="D236" s="9"/>
-      <c r="E236" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="F236" s="9">
-        <v>1212</v>
-      </c>
-      <c r="G236" s="9"/>
-      <c r="H236" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="I236" s="5"/>
-    </row>
-    <row r="237" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A237" s="9" t="s">
-        <v>177</v>
-      </c>
-      <c r="B237" s="9"/>
-      <c r="C237" s="9"/>
-      <c r="D237" s="9"/>
-      <c r="E237" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="F237" s="9">
-        <v>1212</v>
-      </c>
-      <c r="G237" s="9"/>
-      <c r="H237" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="I237" s="5"/>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A238" s="9" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="B238" s="9"/>
       <c r="C238" s="9"/>
@@ -4192,10 +4187,11 @@
       <c r="H238" s="9" t="s">
         <v>176</v>
       </c>
+      <c r="I238" s="5"/>
     </row>
     <row r="239" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A239" s="9" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="B239" s="9"/>
       <c r="C239" s="9"/>
@@ -4208,12 +4204,13 @@
       </c>
       <c r="G239" s="9"/>
       <c r="H239" s="9" t="s">
-        <v>196</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="I239" s="5"/>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A240" s="9" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B240" s="9"/>
       <c r="C240" s="9"/>
@@ -4222,16 +4219,16 @@
         <v>125</v>
       </c>
       <c r="F240" s="9">
-        <v>1779</v>
+        <v>1212</v>
       </c>
       <c r="G240" s="9"/>
       <c r="H240" s="9" t="s">
-        <v>197</v>
+        <v>176</v>
       </c>
     </row>
     <row r="241" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A241" s="9" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B241" s="9"/>
       <c r="C241" s="9"/>
@@ -4244,12 +4241,12 @@
       </c>
       <c r="G241" s="9"/>
       <c r="H241" s="9" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="242" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A242" s="9" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="B242" s="9"/>
       <c r="C242" s="9"/>
@@ -4262,20 +4259,56 @@
       </c>
       <c r="G242" s="9"/>
       <c r="H242" s="9" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="243" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A243" s="9" t="s">
-        <v>201</v>
-      </c>
+        <v>191</v>
+      </c>
+      <c r="B243" s="9"/>
+      <c r="C243" s="9"/>
+      <c r="D243" s="9"/>
       <c r="E243" s="9" t="s">
         <v>125</v>
       </c>
       <c r="F243" s="9">
         <v>1212</v>
       </c>
+      <c r="G243" s="9"/>
       <c r="H243" s="9" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="244" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A244" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="B244" s="9"/>
+      <c r="C244" s="9"/>
+      <c r="D244" s="9"/>
+      <c r="E244" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="F244" s="9">
+        <v>1779</v>
+      </c>
+      <c r="G244" s="9"/>
+      <c r="H244" s="9" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="245" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A245" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="E245" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="F245" s="9">
+        <v>1212</v>
+      </c>
+      <c r="H245" s="9" t="s">
         <v>196</v>
       </c>
     </row>
@@ -4285,7 +4318,7 @@
     <sortCondition ref="C14:C9129"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="I128" r:id="rId1"/>
+    <hyperlink ref="I130" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>

</xml_diff>

<commit_message>
Added rough assumptions on pot. harvest for 'Green manure', 'Ley not harvested' and 'Fallow' to account for crop resid emissions
</commit_message>
<xml_diff>
--- a/data/default/CropProduction.xlsx
+++ b/data/default/CropProduction.xlsx
@@ -10,7 +10,7 @@
     <sheet name="default" sheetId="1" r:id="rId1"/>
     <sheet name="references" sheetId="5" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913" iterateDelta="1E-4"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="205">
   <si>
     <t>f_crop</t>
   </si>
@@ -514,12 +514,6 @@
     <t>kg DM</t>
   </si>
   <si>
-    <t>Anta potentiell skörd</t>
-  </si>
-  <si>
-    <t>Skörd från Pierre</t>
-  </si>
-  <si>
     <t>Anta skörd utifrån vall?</t>
   </si>
   <si>
@@ -656,6 +650,15 @@
   </si>
   <si>
     <t>Fraction of below ground residues renewed annually</t>
+  </si>
+  <si>
+    <t>No prod., harvest = potential, assumed as organic ley * 0.5 need to check!!!</t>
+  </si>
+  <si>
+    <t>No prod., harvest = potential, assumed as organic ley need to check!!!</t>
+  </si>
+  <si>
+    <t>No prod., harvest = potential, assumed as ley for grazing need to check!!!</t>
   </si>
 </sst>
 </file>
@@ -1042,7 +1045,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I245"/>
+  <dimension ref="A1:I246"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="30.42578125" customWidth="1"/>
@@ -1123,7 +1126,7 @@
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -1141,7 +1144,7 @@
         <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -1158,7 +1161,7 @@
         <v>1</v>
       </c>
       <c r="G6" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -1176,7 +1179,7 @@
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -1194,7 +1197,7 @@
         <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -1211,7 +1214,7 @@
         <v>1</v>
       </c>
       <c r="G9" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -1228,7 +1231,7 @@
         <v>1</v>
       </c>
       <c r="G10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -1245,7 +1248,7 @@
         <v>1</v>
       </c>
       <c r="G11" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -1262,7 +1265,7 @@
         <v>1</v>
       </c>
       <c r="G12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -1279,10 +1282,10 @@
         <v>0.5</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="I13" t="s">
         <v>109</v>
@@ -1302,17 +1305,17 @@
         <v>0.5</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
       <c r="D15" s="9" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>47</v>
@@ -1321,10 +1324,10 @@
         <v>1</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -1343,7 +1346,7 @@
         <v>1</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H16" s="9"/>
     </row>
@@ -1363,7 +1366,7 @@
         <v>1</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H17" s="9"/>
     </row>
@@ -1383,7 +1386,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H18" s="9"/>
     </row>
@@ -1407,12 +1410,12 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
       <c r="D20" s="9" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E20" s="9" t="s">
         <v>47</v>
@@ -1425,12 +1428,12 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
       <c r="D21" s="9" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>47</v>
@@ -1443,12 +1446,12 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B22" s="9"/>
       <c r="C22" s="9"/>
       <c r="D22" s="9" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E22" s="9" t="s">
         <v>47</v>
@@ -1497,12 +1500,12 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
       <c r="D25" s="9" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>47</v>
@@ -1515,12 +1518,12 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
       <c r="D26" s="9" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E26" s="9" t="s">
         <v>47</v>
@@ -1533,12 +1536,12 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>
       <c r="D27" s="9" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>47</v>
@@ -1641,10 +1644,10 @@
         <v>155</v>
       </c>
       <c r="H33" t="s">
+        <v>168</v>
+      </c>
+      <c r="I33" t="s">
         <v>170</v>
-      </c>
-      <c r="I33" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -1720,12 +1723,12 @@
       </c>
       <c r="H37" s="4"/>
       <c r="I37" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B38" s="3"/>
       <c r="D38" t="s">
@@ -1742,12 +1745,12 @@
       </c>
       <c r="H38" s="4"/>
       <c r="I38" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B39" s="3"/>
       <c r="D39" t="s">
@@ -1764,7 +1767,7 @@
       </c>
       <c r="H39" s="4"/>
       <c r="I39" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -1819,7 +1822,7 @@
       </c>
       <c r="B43" s="4"/>
       <c r="D43" s="4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E43" t="s">
         <v>47</v>
@@ -1899,7 +1902,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
         <v>31</v>
       </c>
@@ -1914,7 +1917,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>37</v>
       </c>
@@ -1928,7 +1931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>52</v>
       </c>
@@ -1942,7 +1945,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>28</v>
       </c>
@@ -1956,7 +1959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>10</v>
       </c>
@@ -1970,7 +1973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>62</v>
       </c>
@@ -1984,7 +1987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>30</v>
       </c>
@@ -1998,7 +2001,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>70</v>
       </c>
@@ -2012,7 +2015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>80</v>
       </c>
@@ -2026,7 +2029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>55</v>
       </c>
@@ -2040,7 +2043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
         <v>61</v>
       </c>
@@ -2054,7 +2057,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
         <v>54</v>
       </c>
@@ -2069,7 +2072,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>69</v>
       </c>
@@ -2083,7 +2086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>59</v>
       </c>
@@ -2097,128 +2100,107 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="B64" s="8"/>
-      <c r="F64" s="4"/>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B64" s="4"/>
+      <c r="E64" t="s">
+        <v>47</v>
+      </c>
+      <c r="F64" s="9">
+        <v>0</v>
+      </c>
+      <c r="H64" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A65" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B65" s="4" t="s">
-        <v>156</v>
-      </c>
+      <c r="A65" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B65" s="4"/>
       <c r="E65" t="s">
         <v>47</v>
       </c>
       <c r="F65" s="9">
         <v>0</v>
       </c>
+      <c r="H65" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A66" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B66" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="F66" s="9"/>
-    </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A67" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B67" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F67" s="9"/>
+      <c r="A66" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B66" s="4"/>
+      <c r="E66" t="s">
+        <v>47</v>
+      </c>
+      <c r="F66" s="9">
+        <v>0</v>
+      </c>
+      <c r="H66" t="s">
+        <v>204</v>
+      </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A68" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B68" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="E68" t="s">
-        <v>47</v>
-      </c>
-      <c r="F68" s="9">
-        <v>0</v>
-      </c>
+      <c r="A68" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B68" s="8"/>
+      <c r="F68" s="4"/>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="E69" t="s">
-        <v>47</v>
-      </c>
-      <c r="F69" s="9">
-        <v>0</v>
-      </c>
+      <c r="F69" s="9"/>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A70" s="4"/>
+      <c r="A70" s="4" t="s">
+        <v>68</v>
+      </c>
       <c r="B70" s="4"/>
-      <c r="F70" s="4"/>
-    </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A71" s="1" t="s">
+      <c r="F70" s="9"/>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A72" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B71" s="1"/>
-      <c r="C71" s="1"/>
-      <c r="D71" s="1"/>
-      <c r="E71" s="1"/>
-      <c r="F71" s="1"/>
-      <c r="G71" s="12"/>
-      <c r="H71" s="1"/>
-      <c r="I71" s="1"/>
-    </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E72" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="F72" t="s">
-        <v>153</v>
-      </c>
-      <c r="G72" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="H72" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="I72" s="9" t="s">
-        <v>161</v>
-      </c>
+      <c r="B72" s="1"/>
+      <c r="C72" s="1"/>
+      <c r="D72" s="1"/>
+      <c r="E72" s="1"/>
+      <c r="F72" s="1"/>
+      <c r="G72" s="12"/>
+      <c r="H72" s="1"/>
+      <c r="I72" s="1"/>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E73" s="9" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="F73" t="s">
         <v>153</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="I73" s="9" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E74" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F74" t="s">
         <v>153</v>
@@ -2227,157 +2209,162 @@
         <v>130</v>
       </c>
       <c r="H74" s="9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I74" s="9" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E75" s="9" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F75" t="s">
         <v>153</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>144</v>
+        <v>152</v>
+      </c>
+      <c r="I75" s="9" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E76" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F76" t="s">
         <v>153</v>
       </c>
       <c r="G76" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H76" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E77" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F77" t="s">
         <v>153</v>
       </c>
       <c r="G77" s="9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H77" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E78" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F78" t="s">
         <v>153</v>
       </c>
       <c r="G78" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H78" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="I78" s="9" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E79" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F79" t="s">
         <v>153</v>
       </c>
       <c r="G79" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H79" s="9" t="s">
-        <v>148</v>
+        <v>147</v>
+      </c>
+      <c r="I79" s="9" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E80" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F80" t="s">
         <v>153</v>
       </c>
       <c r="G80" s="9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H80" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E81" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F81" t="s">
         <v>153</v>
       </c>
       <c r="G81" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H81" s="9" t="s">
-        <v>150</v>
-      </c>
-      <c r="I81" s="9" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E82" s="9" t="s">
-        <v>202</v>
+        <v>139</v>
       </c>
       <c r="F82" t="s">
         <v>153</v>
       </c>
-      <c r="G82" s="9"/>
+      <c r="G82" s="9" t="s">
+        <v>140</v>
+      </c>
       <c r="H82" s="9" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="I82" s="9" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E83" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F83" s="5">
-        <v>0</v>
-      </c>
-      <c r="H83" s="5" t="s">
-        <v>73</v>
+      <c r="E83" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="F83" t="s">
+        <v>153</v>
+      </c>
+      <c r="G83" s="9"/>
+      <c r="H83" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="I83" s="9" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E84" s="5" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="F84" s="5">
         <v>0</v>
       </c>
-      <c r="G84" s="5"/>
       <c r="H84" s="5" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E85" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F85" s="5">
         <v>0</v>
@@ -2389,18 +2376,19 @@
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E86" s="5" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F86" s="5">
         <v>0</v>
       </c>
+      <c r="G86" s="5"/>
       <c r="H86" s="5" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E87" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F87" s="5">
         <v>0</v>
@@ -2411,7 +2399,7 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E88" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F88" s="5">
         <v>0</v>
@@ -2422,19 +2410,18 @@
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E89" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F89" s="5">
         <v>0</v>
       </c>
-      <c r="G89" s="5"/>
       <c r="H89" s="5" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E90" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F90" s="5">
         <v>0</v>
@@ -2446,7 +2433,7 @@
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E91" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F91" s="5">
         <v>0</v>
@@ -2458,7 +2445,7 @@
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E92" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F92" s="5">
         <v>0</v>
@@ -2470,10 +2457,10 @@
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E93" s="5" t="s">
-        <v>202</v>
+        <v>139</v>
       </c>
       <c r="F93" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G93" s="5"/>
       <c r="H93" s="5" t="s">
@@ -2481,58 +2468,50 @@
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F94" s="4"/>
+      <c r="E94" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="F94" s="5">
+        <v>1</v>
+      </c>
+      <c r="G94" s="5"/>
+      <c r="H94" s="5" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A95" s="1" t="s">
+      <c r="F95" s="4"/>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A96" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B95" s="1"/>
-      <c r="C95" s="1"/>
-      <c r="D95" s="1"/>
-      <c r="E95" s="2"/>
-      <c r="F95" s="2"/>
-      <c r="G95" s="2" t="s">
+      <c r="B96" s="1"/>
+      <c r="C96" s="1"/>
+      <c r="D96" s="1"/>
+      <c r="E96" s="2"/>
+      <c r="F96" s="2"/>
+      <c r="G96" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="H95" s="2"/>
-      <c r="I95" s="2"/>
-    </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E96" s="5" t="s">
+      <c r="H96" s="2"/>
+      <c r="I96" s="2"/>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E97" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="F96" s="5">
+      <c r="F97" s="5">
         <v>0</v>
       </c>
-      <c r="G96" s="5"/>
-      <c r="H96" s="5" t="s">
+      <c r="G97" s="5"/>
+      <c r="H97" s="5" t="s">
         <v>73</v>
-      </c>
-    </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>42</v>
-      </c>
-      <c r="C97" t="s">
-        <v>11</v>
-      </c>
-      <c r="D97" t="s">
-        <v>44</v>
-      </c>
-      <c r="E97" t="s">
-        <v>107</v>
-      </c>
-      <c r="F97">
-        <v>210</v>
-      </c>
-      <c r="I97" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C98" t="s">
         <v>11</v>
@@ -2543,8 +2522,8 @@
       <c r="E98" t="s">
         <v>107</v>
       </c>
-      <c r="F98" s="9">
-        <v>235</v>
+      <c r="F98">
+        <v>210</v>
       </c>
       <c r="I98" t="s">
         <v>108</v>
@@ -2552,10 +2531,10 @@
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C99" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D99" t="s">
         <v>44</v>
@@ -2564,15 +2543,15 @@
         <v>107</v>
       </c>
       <c r="F99" s="9">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="I99" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C100" t="s">
         <v>12</v>
@@ -2592,33 +2571,36 @@
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>34</v>
+        <v>41</v>
+      </c>
+      <c r="C101" t="s">
+        <v>12</v>
       </c>
       <c r="D101" t="s">
-        <v>75</v>
+        <v>44</v>
       </c>
       <c r="E101" t="s">
         <v>107</v>
       </c>
       <c r="F101" s="9">
-        <v>140</v>
+        <v>230</v>
       </c>
       <c r="I101" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="D102" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E102" t="s">
         <v>107</v>
       </c>
       <c r="F102" s="9">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="I102" t="s">
         <v>108</v>
@@ -2626,10 +2608,7 @@
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>13</v>
-      </c>
-      <c r="C103" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D103" t="s">
         <v>72</v>
@@ -2646,10 +2625,10 @@
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C104" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D104" t="s">
         <v>72</v>
@@ -2658,15 +2637,15 @@
         <v>107</v>
       </c>
       <c r="F104" s="9">
-        <v>210</v>
-      </c>
-      <c r="H104" t="s">
-        <v>114</v>
+        <v>180</v>
+      </c>
+      <c r="I104" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C105" t="s">
         <v>12</v>
@@ -2680,28 +2659,28 @@
       <c r="F105" s="9">
         <v>210</v>
       </c>
-      <c r="I105" t="s">
-        <v>109</v>
+      <c r="H105" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="C106" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D106" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E106" t="s">
         <v>107</v>
       </c>
       <c r="F106" s="9">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="I106" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -2709,7 +2688,7 @@
         <v>27</v>
       </c>
       <c r="C107" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D107" t="s">
         <v>76</v>
@@ -2718,32 +2697,35 @@
         <v>107</v>
       </c>
       <c r="F107" s="9">
-        <v>230</v>
+        <v>190</v>
       </c>
       <c r="I107" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>40</v>
+        <v>27</v>
+      </c>
+      <c r="C108" t="s">
+        <v>12</v>
       </c>
       <c r="D108" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="E108" t="s">
         <v>107</v>
       </c>
-      <c r="F108">
-        <v>180</v>
+      <c r="F108" s="9">
+        <v>230</v>
       </c>
       <c r="I108" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D109" t="s">
         <v>83</v>
@@ -2754,34 +2736,32 @@
       <c r="F109">
         <v>180</v>
       </c>
-      <c r="H109" t="s">
+      <c r="I109" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>39</v>
+      </c>
+      <c r="D110" t="s">
+        <v>83</v>
+      </c>
+      <c r="E110" t="s">
+        <v>107</v>
+      </c>
+      <c r="F110">
+        <v>180</v>
+      </c>
+      <c r="H110" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A110" s="4" t="s">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A111" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B110" s="4"/>
-    </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A111" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B111" s="9"/>
-      <c r="C111" s="9"/>
-      <c r="D111" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="E111" t="s">
-        <v>107</v>
-      </c>
-      <c r="F111" s="9">
-        <v>100</v>
-      </c>
-      <c r="I111" t="s">
-        <v>109</v>
-      </c>
+      <c r="B111" s="4"/>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" s="9" t="s">
@@ -2790,56 +2770,52 @@
       <c r="B112" s="9"/>
       <c r="C112" s="9"/>
       <c r="D112" s="9" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E112" t="s">
         <v>107</v>
       </c>
       <c r="F112" s="9">
+        <v>100</v>
+      </c>
+      <c r="I112" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A113" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B113" s="9"/>
+      <c r="C113" s="9"/>
+      <c r="D113" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="E113" t="s">
+        <v>107</v>
+      </c>
+      <c r="F113" s="9">
         <v>110</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A113" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="B113" s="5"/>
-      <c r="C113" s="5"/>
-      <c r="D113" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="E113" s="5" t="s">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A114" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B114" s="5"/>
+      <c r="C114" s="5"/>
+      <c r="D114" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E114" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="F113" s="5">
+      <c r="F114" s="5">
         <v>0</v>
       </c>
-      <c r="G113" s="5"/>
-      <c r="H113" s="5" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
-        <v>32</v>
-      </c>
-      <c r="C114" t="s">
-        <v>11</v>
-      </c>
-      <c r="D114" t="s">
-        <v>84</v>
-      </c>
-      <c r="E114" t="s">
-        <v>107</v>
-      </c>
-      <c r="F114">
-        <v>20</v>
-      </c>
-      <c r="H114" t="s">
-        <v>111</v>
-      </c>
-      <c r="I114" t="s">
-        <v>108</v>
+      <c r="G114" s="5"/>
+      <c r="H114" s="5" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -2847,7 +2823,7 @@
         <v>32</v>
       </c>
       <c r="C115" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D115" t="s">
         <v>84</v>
@@ -2856,47 +2832,50 @@
         <v>107</v>
       </c>
       <c r="F115">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H115" t="s">
         <v>111</v>
       </c>
       <c r="I115" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>32</v>
+      </c>
+      <c r="C116" t="s">
+        <v>12</v>
+      </c>
+      <c r="D116" t="s">
+        <v>84</v>
+      </c>
+      <c r="E116" t="s">
+        <v>107</v>
+      </c>
+      <c r="F116">
+        <v>21</v>
+      </c>
+      <c r="H116" t="s">
+        <v>111</v>
+      </c>
+      <c r="I116" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A116" s="4" t="s">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A117" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B116" s="4"/>
-    </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>15</v>
-      </c>
-      <c r="C117" t="s">
-        <v>11</v>
-      </c>
-      <c r="D117" t="s">
-        <v>85</v>
-      </c>
-      <c r="E117" t="s">
-        <v>107</v>
-      </c>
-      <c r="F117">
-        <v>9</v>
-      </c>
-      <c r="I117" t="s">
-        <v>108</v>
-      </c>
+      <c r="B117" s="4"/>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>15</v>
       </c>
       <c r="C118" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D118" t="s">
         <v>85</v>
@@ -2905,33 +2884,41 @@
         <v>107</v>
       </c>
       <c r="F118">
+        <v>9</v>
+      </c>
+      <c r="I118" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>15</v>
+      </c>
+      <c r="C119" t="s">
+        <v>12</v>
+      </c>
+      <c r="D119" t="s">
+        <v>85</v>
+      </c>
+      <c r="E119" t="s">
+        <v>107</v>
+      </c>
+      <c r="F119">
         <v>9.5</v>
       </c>
-      <c r="I118" t="s">
+      <c r="I119" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A119" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B119" s="4"/>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="B120" s="5"/>
-      <c r="C120" s="5"/>
-      <c r="D120" s="5"/>
-      <c r="E120" s="5"/>
-      <c r="F120" s="5"/>
-      <c r="G120" s="5"/>
-      <c r="H120" s="5"/>
+        <v>74</v>
+      </c>
+      <c r="B120" s="4"/>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" s="4" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="B121" s="5"/>
       <c r="C121" s="5"/>
@@ -2943,7 +2930,7 @@
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B122" s="5"/>
       <c r="C122" s="5"/>
@@ -2954,31 +2941,23 @@
       <c r="H122" s="5"/>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
-        <v>67</v>
-      </c>
-      <c r="C123" t="s">
-        <v>11</v>
-      </c>
-      <c r="D123" t="s">
-        <v>82</v>
-      </c>
-      <c r="E123" t="s">
-        <v>107</v>
-      </c>
-      <c r="F123">
-        <v>0.33</v>
-      </c>
-      <c r="I123" t="s">
-        <v>108</v>
-      </c>
+      <c r="A123" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B123" s="5"/>
+      <c r="C123" s="5"/>
+      <c r="D123" s="5"/>
+      <c r="E123" s="5"/>
+      <c r="F123" s="5"/>
+      <c r="G123" s="5"/>
+      <c r="H123" s="5"/>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>67</v>
       </c>
       <c r="C124" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D124" t="s">
         <v>82</v>
@@ -2987,46 +2966,56 @@
         <v>107</v>
       </c>
       <c r="F124">
+        <v>0.33</v>
+      </c>
+      <c r="I124" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>67</v>
+      </c>
+      <c r="C125" t="s">
+        <v>12</v>
+      </c>
+      <c r="D125" t="s">
+        <v>82</v>
+      </c>
+      <c r="E125" t="s">
+        <v>107</v>
+      </c>
+      <c r="F125">
         <f>(5+0.4)/2</f>
         <v>2.7</v>
       </c>
-      <c r="H124" t="s">
+      <c r="H125" t="s">
         <v>110</v>
       </c>
-      <c r="I124" t="s">
+      <c r="I125" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
         <v>66</v>
       </c>
-      <c r="D125" t="s">
+      <c r="D126" t="s">
         <v>82</v>
       </c>
-      <c r="E125" t="s">
+      <c r="E126" t="s">
         <v>107</v>
       </c>
-      <c r="F125">
+      <c r="F126">
         <v>0.67</v>
       </c>
-      <c r="I125" t="s">
+      <c r="I126" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A126" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="B126" s="5"/>
-      <c r="C126" s="5"/>
-      <c r="D126" s="5"/>
-      <c r="E126" s="5"/>
-      <c r="F126" s="5"/>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" s="4" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B127" s="5"/>
       <c r="C127" s="5"/>
@@ -3036,7 +3025,7 @@
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" s="4" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B128" s="5"/>
       <c r="C128" s="5"/>
@@ -3045,112 +3034,101 @@
       <c r="F128" s="5"/>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A129" t="s">
+      <c r="A129" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B129" s="5"/>
+      <c r="C129" s="5"/>
+      <c r="D129" s="5"/>
+      <c r="E129" s="5"/>
+      <c r="F129" s="5"/>
+    </row>
+    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
         <v>64</v>
       </c>
-      <c r="D129" t="s">
+      <c r="D130" t="s">
         <v>78</v>
       </c>
-      <c r="E129" t="s">
+      <c r="E130" t="s">
         <v>107</v>
       </c>
-      <c r="F129">
+      <c r="F130">
         <f>900+1800</f>
         <v>2700</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A130" t="s">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
         <v>63</v>
       </c>
-      <c r="D130" t="s">
+      <c r="D131" t="s">
         <v>77</v>
       </c>
-      <c r="E130" t="s">
+      <c r="E131" t="s">
         <v>107</v>
       </c>
-      <c r="F130">
+      <c r="F131">
         <v>2000</v>
       </c>
-      <c r="H130" t="s">
+      <c r="H131" t="s">
         <v>112</v>
       </c>
-      <c r="I130" s="10" t="s">
+      <c r="I131" s="10" t="s">
         <v>113</v>
-      </c>
-    </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A131" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B131" s="4"/>
-      <c r="H131" s="4" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="B132" s="4"/>
-      <c r="D132" t="s">
-        <v>95</v>
-      </c>
-      <c r="E132" t="s">
-        <v>107</v>
-      </c>
-      <c r="F132" s="4">
-        <v>5</v>
+      <c r="H132" s="4" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" s="4" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B133" s="4"/>
+      <c r="D133" t="s">
+        <v>95</v>
+      </c>
+      <c r="E133" t="s">
+        <v>107</v>
+      </c>
+      <c r="F133" s="4">
+        <v>5</v>
+      </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" s="4" t="s">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="B134" s="4"/>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" s="4" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B135" s="4"/>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B136" s="4"/>
+    </row>
+    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A137" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B136" s="4"/>
-    </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A137" s="9" t="s">
-        <v>22</v>
-      </c>
       <c r="B137" s="4"/>
-      <c r="D137" t="s">
-        <v>95</v>
-      </c>
-      <c r="E137" t="s">
-        <v>107</v>
-      </c>
-      <c r="F137">
-        <v>7</v>
-      </c>
-      <c r="H137" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="I137" t="s">
-        <v>108</v>
-      </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B138" s="4"/>
       <c r="D138" t="s">
@@ -3160,60 +3138,66 @@
         <v>107</v>
       </c>
       <c r="F138">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H138" s="4" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I138" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A139" s="4" t="s">
-        <v>56</v>
+      <c r="A139" s="9" t="s">
+        <v>23</v>
       </c>
       <c r="B139" s="4"/>
+      <c r="D139" t="s">
+        <v>95</v>
+      </c>
+      <c r="E139" t="s">
+        <v>107</v>
+      </c>
+      <c r="F139">
+        <v>4</v>
+      </c>
       <c r="H139" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
+      </c>
+      <c r="I139" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="4" t="s">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="B140" s="4"/>
+      <c r="H140" s="4" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" s="4" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="B141" s="4"/>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B142" s="4"/>
+    </row>
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A143" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B142" s="4"/>
-    </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A143" s="9" t="s">
+      <c r="B143" s="4"/>
+    </row>
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A144" s="9" t="s">
         <v>36</v>
-      </c>
-      <c r="B143" s="9"/>
-      <c r="C143" s="9"/>
-      <c r="D143" s="9"/>
-      <c r="E143" s="9"/>
-      <c r="F143" s="3">
-        <v>0</v>
-      </c>
-      <c r="H143" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A144" s="3" t="s">
-        <v>173</v>
       </c>
       <c r="B144" s="9"/>
       <c r="C144" s="9"/>
@@ -3223,27 +3207,27 @@
         <v>0</v>
       </c>
       <c r="H144" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A145" s="3" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B145" s="9"/>
       <c r="C145" s="9"/>
       <c r="D145" s="9"/>
       <c r="E145" s="9"/>
-      <c r="F145" s="9">
+      <c r="F145" s="3">
         <v>0</v>
       </c>
       <c r="H145" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A146" s="9" t="s">
-        <v>35</v>
+      <c r="A146" s="3" t="s">
+        <v>172</v>
       </c>
       <c r="B146" s="9"/>
       <c r="C146" s="9"/>
@@ -3253,376 +3237,380 @@
         <v>0</v>
       </c>
       <c r="H146" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A147" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B147" s="4"/>
+      <c r="A147" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B147" s="9"/>
+      <c r="C147" s="9"/>
+      <c r="D147" s="9"/>
+      <c r="E147" s="9"/>
+      <c r="F147" s="9">
+        <v>0</v>
+      </c>
+      <c r="H147" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A148" s="4" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="B148" s="4"/>
     </row>
     <row r="149" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A149" s="4" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B149" s="4"/>
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A150" s="4" t="s">
-        <v>21</v>
+        <v>60</v>
       </c>
       <c r="B150" s="4"/>
     </row>
     <row r="151" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A151" s="4" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B151" s="4"/>
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A152" s="4" t="s">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="B152" s="4"/>
     </row>
     <row r="153" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A153" s="4" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="B153" s="4"/>
     </row>
     <row r="154" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A154" s="4" t="s">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="B154" s="4"/>
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A155" s="4" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B155" s="4"/>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A156" s="4" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B156" s="4"/>
     </row>
     <row r="157" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A157" s="4" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="B157" s="4"/>
     </row>
     <row r="158" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A158" s="4" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="B158" s="4"/>
     </row>
     <row r="159" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A159" s="4" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="B159" s="4"/>
     </row>
     <row r="160" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A160" s="4" t="s">
-        <v>62</v>
+        <v>10</v>
       </c>
       <c r="B160" s="4"/>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" s="4" t="s">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="B161" s="4"/>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" s="4" t="s">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="B162" s="4"/>
-      <c r="G162" s="4" t="s">
-        <v>166</v>
-      </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A163" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="B163" s="4"/>
       <c r="G163" s="4" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" s="4" t="s">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="B164" s="4"/>
       <c r="G164" s="4" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A165" s="4" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B165" s="4"/>
       <c r="G165" s="4" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A166" s="4" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B166" s="4"/>
       <c r="G166" s="4" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A167" s="4" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="B167" s="4"/>
       <c r="G167" s="4" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A168" s="4" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="B168" s="4"/>
       <c r="G168" s="4" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F169" s="4"/>
+      <c r="A169" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B169" s="4"/>
+      <c r="G169" s="4" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A170" s="1" t="s">
+      <c r="F170" s="4"/>
+    </row>
+    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A171" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B170" s="1"/>
-      <c r="C170" s="1"/>
-      <c r="D170" s="1"/>
-      <c r="E170" s="2"/>
-      <c r="F170" s="2"/>
-      <c r="G170" s="2"/>
-      <c r="H170" s="2"/>
-      <c r="I170" s="2"/>
-    </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B171" t="s">
-        <v>49</v>
-      </c>
-      <c r="E171" t="s">
-        <v>122</v>
-      </c>
-      <c r="F171" s="11">
-        <f>1/7*100</f>
-        <v>14.285714285714285</v>
-      </c>
-      <c r="G171" t="s">
-        <v>123</v>
-      </c>
+      <c r="B171" s="1"/>
+      <c r="C171" s="1"/>
+      <c r="D171" s="1"/>
+      <c r="E171" s="2"/>
+      <c r="F171" s="2"/>
+      <c r="G171" s="2"/>
+      <c r="H171" s="2"/>
+      <c r="I171" s="2"/>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B172" t="s">
         <v>49</v>
       </c>
-      <c r="C172" t="s">
-        <v>12</v>
-      </c>
       <c r="E172" t="s">
         <v>122</v>
       </c>
-      <c r="F172" s="4">
+      <c r="F172" s="11">
+        <f>1/7*100</f>
+        <v>14.285714285714285</v>
+      </c>
+      <c r="G172" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B173" t="s">
+        <v>49</v>
+      </c>
+      <c r="C173" t="s">
+        <v>12</v>
+      </c>
+      <c r="E173" t="s">
+        <v>122</v>
+      </c>
+      <c r="F173" s="4">
         <f>1/8*100</f>
         <v>12.5</v>
       </c>
-      <c r="G172" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B173" t="s">
-        <v>48</v>
-      </c>
-      <c r="E173" t="s">
-        <v>122</v>
-      </c>
-      <c r="F173" s="11">
-        <f>1/6*100</f>
-        <v>16.666666666666664</v>
-      </c>
       <c r="G173" t="s">
         <v>123</v>
-      </c>
-      <c r="I173" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B174" t="s">
         <v>48</v>
       </c>
-      <c r="C174" t="s">
-        <v>12</v>
-      </c>
       <c r="E174" t="s">
         <v>122</v>
       </c>
       <c r="F174" s="11">
+        <f>1/6*100</f>
+        <v>16.666666666666664</v>
+      </c>
+      <c r="G174" t="s">
+        <v>123</v>
+      </c>
+      <c r="I174" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B175" t="s">
+        <v>48</v>
+      </c>
+      <c r="C175" t="s">
+        <v>12</v>
+      </c>
+      <c r="E175" t="s">
+        <v>122</v>
+      </c>
+      <c r="F175" s="11">
         <f>1/10*100</f>
         <v>10</v>
       </c>
-      <c r="G174" t="s">
+      <c r="G175" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F175" s="4"/>
-    </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A176" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="B176" s="1"/>
-      <c r="C176" s="1"/>
-      <c r="D176" s="1"/>
-      <c r="E176" s="2"/>
-      <c r="F176" s="2"/>
-      <c r="G176" s="2" t="s">
+      <c r="F176" s="4"/>
+    </row>
+    <row r="177" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A177" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="H176" s="2"/>
-      <c r="I176" s="2"/>
-    </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E177" s="5" t="s">
+      <c r="B177" s="1"/>
+      <c r="C177" s="1"/>
+      <c r="D177" s="1"/>
+      <c r="E177" s="2"/>
+      <c r="F177" s="2"/>
+      <c r="G177" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="H177" s="2"/>
+      <c r="I177" s="2"/>
+    </row>
+    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E178" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F177" s="5">
+      <c r="F178" s="5">
         <v>0</v>
       </c>
-      <c r="G177" s="5"/>
-      <c r="H177" s="5" t="s">
+      <c r="G178" s="5"/>
+      <c r="H178" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E178" t="s">
+    <row r="179" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E179" t="s">
         <v>7</v>
       </c>
-      <c r="F178" t="s">
+      <c r="F179" t="s">
         <v>154</v>
       </c>
-      <c r="H178" t="s">
+      <c r="H179" t="s">
         <v>124</v>
       </c>
-      <c r="I178" t="s">
+      <c r="I179" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A180" s="1" t="s">
+    <row r="181" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A181" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B180" s="1"/>
-      <c r="C180" s="1"/>
-      <c r="D180" s="1"/>
-      <c r="E180" s="2"/>
-      <c r="F180" s="2"/>
-      <c r="G180" s="2"/>
-      <c r="H180" s="2"/>
-      <c r="I180" s="2"/>
-    </row>
-    <row r="182" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A182" t="s">
-        <v>10</v>
-      </c>
-      <c r="E182" t="s">
-        <v>125</v>
-      </c>
-      <c r="F182">
-        <v>1507</v>
-      </c>
-      <c r="G182" t="s">
-        <v>168</v>
-      </c>
+      <c r="B181" s="1"/>
+      <c r="C181" s="1"/>
+      <c r="D181" s="1"/>
+      <c r="E181" s="2"/>
+      <c r="F181" s="2"/>
+      <c r="G181" s="2"/>
+      <c r="H181" s="2"/>
+      <c r="I181" s="2"/>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E183" t="s">
         <v>125</v>
       </c>
       <c r="F183">
-        <v>979</v>
+        <v>1507</v>
+      </c>
+      <c r="G183" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E184" t="s">
         <v>125</v>
       </c>
       <c r="F184">
-        <v>1211</v>
+        <v>979</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E185" t="s">
         <v>125</v>
       </c>
       <c r="F185">
-        <v>1779</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="E186" t="s">
         <v>125</v>
       </c>
       <c r="F186">
-        <v>1092</v>
+        <v>1779</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E187" t="s">
         <v>125</v>
       </c>
       <c r="F187">
-        <v>1015</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="188" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="E188" t="s">
         <v>125</v>
@@ -3633,51 +3621,51 @@
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>17</v>
+        <v>50</v>
       </c>
       <c r="E189" t="s">
         <v>125</v>
       </c>
       <c r="F189">
-        <v>648</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E190" t="s">
         <v>125</v>
       </c>
       <c r="F190">
-        <v>1185</v>
+        <v>648</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="E191" t="s">
         <v>125</v>
       </c>
       <c r="F191">
-        <v>1015</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="192" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>52</v>
+        <v>80</v>
       </c>
       <c r="E192" t="s">
         <v>125</v>
       </c>
       <c r="F192">
-        <v>944</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E193" t="s">
         <v>125</v>
@@ -3688,84 +3676,84 @@
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="E194" t="s">
         <v>125</v>
       </c>
       <c r="F194">
-        <v>628</v>
+        <v>944</v>
       </c>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E195" t="s">
         <v>125</v>
       </c>
       <c r="F195">
-        <v>1015</v>
+        <v>628</v>
       </c>
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E196" t="s">
         <v>125</v>
       </c>
       <c r="F196">
-        <v>1185</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="E197" t="s">
         <v>125</v>
       </c>
       <c r="F197">
-        <v>1092</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="E198" t="s">
         <v>125</v>
       </c>
       <c r="F198">
-        <v>1015</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E199" t="s">
         <v>125</v>
       </c>
       <c r="F199">
-        <v>1474</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="E200" t="s">
         <v>125</v>
       </c>
       <c r="F200">
-        <v>628</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E201" t="s">
         <v>125</v>
@@ -3776,40 +3764,40 @@
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E202" t="s">
         <v>125</v>
       </c>
       <c r="F202">
-        <v>1073</v>
+        <v>628</v>
       </c>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="E203" t="s">
         <v>125</v>
       </c>
       <c r="F203">
-        <v>628</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="E204" t="s">
         <v>125</v>
       </c>
       <c r="F204">
-        <v>1486</v>
+        <v>628</v>
       </c>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E205" t="s">
         <v>125</v>
@@ -3820,95 +3808,95 @@
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="E206" t="s">
         <v>125</v>
       </c>
       <c r="F206">
-        <v>648</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>27</v>
+        <v>57</v>
       </c>
       <c r="E207" t="s">
         <v>125</v>
       </c>
       <c r="F207">
-        <v>979</v>
+        <v>648</v>
       </c>
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="E208" t="s">
         <v>125</v>
       </c>
       <c r="F208">
-        <v>1073</v>
+        <v>979</v>
       </c>
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="E209" t="s">
         <v>125</v>
       </c>
       <c r="F209">
-        <v>944</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="210" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="E210" t="s">
         <v>125</v>
       </c>
       <c r="F210">
-        <v>1015</v>
+        <v>944</v>
       </c>
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="E211" t="s">
         <v>125</v>
       </c>
       <c r="F211">
-        <v>766</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="212" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E212" t="s">
         <v>125</v>
       </c>
       <c r="F212">
-        <v>1507</v>
+        <v>766</v>
       </c>
     </row>
     <row r="213" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="E213" t="s">
         <v>125</v>
       </c>
       <c r="F213">
-        <v>1015</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="214" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="E214" t="s">
         <v>125</v>
@@ -3919,51 +3907,51 @@
     </row>
     <row r="215" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="E215" t="s">
         <v>125</v>
       </c>
       <c r="F215">
-        <v>1185</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="216" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E216" t="s">
         <v>125</v>
       </c>
       <c r="F216">
-        <v>1507</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="217" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="E217" t="s">
         <v>125</v>
       </c>
       <c r="F217">
-        <v>1211</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="218" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E218" t="s">
         <v>125</v>
       </c>
       <c r="F218">
-        <v>1569</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="E219" t="s">
         <v>125</v>
@@ -3974,73 +3962,73 @@
     </row>
     <row r="220" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E220" t="s">
         <v>125</v>
       </c>
       <c r="F220">
-        <v>766</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="221" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E221" t="s">
         <v>125</v>
       </c>
       <c r="F221">
-        <v>1185</v>
+        <v>766</v>
       </c>
     </row>
     <row r="222" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E222" t="s">
         <v>125</v>
       </c>
       <c r="F222">
-        <v>1015</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="223" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E223" t="s">
         <v>125</v>
       </c>
       <c r="F223">
-        <v>1211</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="224" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="E224" t="s">
         <v>125</v>
       </c>
       <c r="F224">
-        <v>1015</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E225" t="s">
         <v>125</v>
       </c>
       <c r="F225">
-        <v>628</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="226" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E226" t="s">
         <v>125</v>
@@ -4050,8 +4038,8 @@
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A227" s="3" t="s">
-        <v>173</v>
+      <c r="A227" t="s">
+        <v>36</v>
       </c>
       <c r="E227" t="s">
         <v>125</v>
@@ -4062,7 +4050,7 @@
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A228" s="3" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E228" t="s">
         <v>125</v>
@@ -4072,30 +4060,30 @@
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A229" t="s">
-        <v>68</v>
+      <c r="A229" s="3" t="s">
+        <v>172</v>
       </c>
       <c r="E229" t="s">
         <v>125</v>
       </c>
       <c r="F229">
-        <v>1224</v>
+        <v>628</v>
       </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>37</v>
+        <v>68</v>
       </c>
       <c r="E230" t="s">
         <v>125</v>
       </c>
       <c r="F230">
-        <v>1015</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="E231" t="s">
         <v>125</v>
@@ -4106,40 +4094,40 @@
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="E232" t="s">
         <v>125</v>
       </c>
       <c r="F232">
-        <v>1721</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>70</v>
+        <v>38</v>
       </c>
       <c r="E233" t="s">
         <v>125</v>
       </c>
       <c r="F233">
-        <v>1015</v>
+        <v>1721</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="E234" t="s">
         <v>125</v>
       </c>
       <c r="F234">
-        <v>1211</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E235" t="s">
         <v>125</v>
@@ -4150,48 +4138,40 @@
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E236" t="s">
         <v>125</v>
       </c>
       <c r="F236">
-        <v>979</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
+        <v>41</v>
+      </c>
+      <c r="E237" t="s">
+        <v>125</v>
+      </c>
+      <c r="F237">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="238" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A238" t="s">
         <v>42</v>
       </c>
-      <c r="E237" t="s">
-        <v>125</v>
-      </c>
-      <c r="F237">
+      <c r="E238" t="s">
+        <v>125</v>
+      </c>
+      <c r="F238">
         <v>1015</v>
       </c>
-    </row>
-    <row r="238" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A238" s="9" t="s">
-        <v>175</v>
-      </c>
-      <c r="B238" s="9"/>
-      <c r="C238" s="9"/>
-      <c r="D238" s="9"/>
-      <c r="E238" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="F238" s="9">
-        <v>1212</v>
-      </c>
-      <c r="G238" s="9"/>
-      <c r="H238" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="I238" s="5"/>
     </row>
     <row r="239" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A239" s="9" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B239" s="9"/>
       <c r="C239" s="9"/>
@@ -4204,13 +4184,13 @@
       </c>
       <c r="G239" s="9"/>
       <c r="H239" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="I239" s="5"/>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A240" s="9" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="B240" s="9"/>
       <c r="C240" s="9"/>
@@ -4223,12 +4203,13 @@
       </c>
       <c r="G240" s="9"/>
       <c r="H240" s="9" t="s">
-        <v>176</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="I240" s="5"/>
     </row>
     <row r="241" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A241" s="9" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B241" s="9"/>
       <c r="C241" s="9"/>
@@ -4241,7 +4222,7 @@
       </c>
       <c r="G241" s="9"/>
       <c r="H241" s="9" t="s">
-        <v>196</v>
+        <v>174</v>
       </c>
     </row>
     <row r="242" spans="1:8" x14ac:dyDescent="0.25">
@@ -4255,16 +4236,16 @@
         <v>125</v>
       </c>
       <c r="F242" s="9">
-        <v>1779</v>
+        <v>1212</v>
       </c>
       <c r="G242" s="9"/>
       <c r="H242" s="9" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="243" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A243" s="9" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="B243" s="9"/>
       <c r="C243" s="9"/>
@@ -4273,16 +4254,16 @@
         <v>125</v>
       </c>
       <c r="F243" s="9">
-        <v>1212</v>
+        <v>1779</v>
       </c>
       <c r="G243" s="9"/>
       <c r="H243" s="9" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="244" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A244" s="9" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B244" s="9"/>
       <c r="C244" s="9"/>
@@ -4291,25 +4272,43 @@
         <v>125</v>
       </c>
       <c r="F244" s="9">
-        <v>1779</v>
+        <v>1212</v>
       </c>
       <c r="G244" s="9"/>
       <c r="H244" s="9" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="245" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A245" s="9" t="s">
-        <v>201</v>
-      </c>
+        <v>191</v>
+      </c>
+      <c r="B245" s="9"/>
+      <c r="C245" s="9"/>
+      <c r="D245" s="9"/>
       <c r="E245" s="9" t="s">
         <v>125</v>
       </c>
       <c r="F245" s="9">
+        <v>1779</v>
+      </c>
+      <c r="G245" s="9"/>
+      <c r="H245" s="9" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="246" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A246" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="E246" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="F246" s="9">
         <v>1212</v>
       </c>
-      <c r="H245" s="9" t="s">
-        <v>196</v>
+      <c r="H246" s="9" t="s">
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -4318,7 +4317,7 @@
     <sortCondition ref="C14:C9129"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="I130" r:id="rId1"/>
+    <hyperlink ref="I131" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
@@ -4332,22 +4331,22 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
No GDD constraint for 'Green manure' an 'Energy grass'
</commit_message>
<xml_diff>
--- a/data/default/CropProduction.xlsx
+++ b/data/default/CropProduction.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="665" uniqueCount="206">
   <si>
     <t>f_crop</t>
   </si>
@@ -659,6 +659,9 @@
   </si>
   <si>
     <t>No prod., harvest = potential, assumed as ley for grazing need to check!!!</t>
+  </si>
+  <si>
+    <t>Same as ley for fodder</t>
   </si>
 </sst>
 </file>
@@ -3663,7 +3666,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>52</v>
       </c>
@@ -3674,7 +3677,7 @@
         <v>944</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>53</v>
       </c>
@@ -3682,10 +3685,13 @@
         <v>125</v>
       </c>
       <c r="F194">
-        <v>944</v>
-      </c>
-    </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
+        <v>628</v>
+      </c>
+      <c r="H194" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>18</v>
       </c>
@@ -3696,7 +3702,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>19</v>
       </c>
@@ -3704,10 +3710,13 @@
         <v>125</v>
       </c>
       <c r="F196">
-        <v>1015</v>
-      </c>
-    </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
+        <v>628</v>
+      </c>
+      <c r="H196" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>20</v>
       </c>
@@ -3718,7 +3727,7 @@
         <v>1185</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>54</v>
       </c>
@@ -3729,7 +3738,7 @@
         <v>1092</v>
       </c>
     </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>21</v>
       </c>
@@ -3740,7 +3749,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>55</v>
       </c>
@@ -3751,7 +3760,7 @@
         <v>1474</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>22</v>
       </c>
@@ -3762,7 +3771,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>23</v>
       </c>
@@ -3773,7 +3782,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>24</v>
       </c>
@@ -3784,7 +3793,7 @@
         <v>1073</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>56</v>
       </c>
@@ -3795,7 +3804,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>25</v>
       </c>
@@ -3806,7 +3815,7 @@
         <v>1486</v>
       </c>
     </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>26</v>
       </c>
@@ -3817,7 +3826,7 @@
         <v>1486</v>
       </c>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>57</v>
       </c>
@@ -3828,7 +3837,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Import parameters for crop residue C from csv
</commit_message>
<xml_diff>
--- a/data/default/CropProduction.xlsx
+++ b/data/default/CropProduction.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="665" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="211">
   <si>
     <t>f_crop</t>
   </si>
@@ -662,6 +662,21 @@
   </si>
   <si>
     <t>Same as ley for fodder</t>
+  </si>
+  <si>
+    <t>ag_resid_C</t>
+  </si>
+  <si>
+    <t>bg_resid_C</t>
+  </si>
+  <si>
+    <t>kg C/kg DM</t>
+  </si>
+  <si>
+    <t>Carbon in above ground residues</t>
+  </si>
+  <si>
+    <t>Carbon in below ground residues</t>
   </si>
 </sst>
 </file>
@@ -1048,7 +1063,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I246"/>
+  <dimension ref="A1:I250"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="30.42578125" customWidth="1"/>
@@ -2308,7 +2323,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="81" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E81" s="9" t="s">
         <v>138</v>
       </c>
@@ -2322,98 +2337,105 @@
         <v>149</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="82" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E82" s="9" t="s">
-        <v>139</v>
+        <v>206</v>
       </c>
       <c r="F82" t="s">
         <v>153</v>
       </c>
       <c r="G82" s="9" t="s">
-        <v>140</v>
+        <v>208</v>
       </c>
       <c r="H82" s="9" t="s">
-        <v>150</v>
-      </c>
-      <c r="I82" s="9" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="83" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E83" s="9" t="s">
-        <v>200</v>
+        <v>139</v>
       </c>
       <c r="F83" t="s">
         <v>153</v>
       </c>
-      <c r="G83" s="9"/>
+      <c r="G83" s="9" t="s">
+        <v>140</v>
+      </c>
       <c r="H83" s="9" t="s">
-        <v>201</v>
+        <v>150</v>
       </c>
       <c r="I83" s="9" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E84" s="5" t="s">
+    <row r="84" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E84" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="F84" t="s">
+        <v>153</v>
+      </c>
+      <c r="G84" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="H84" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="I84" s="9"/>
+    </row>
+    <row r="85" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E85" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="F85" t="s">
+        <v>153</v>
+      </c>
+      <c r="G85" s="9"/>
+      <c r="H85" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="I85" s="9" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="86" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E86" s="5" t="s">
         <v>131</v>
-      </c>
-      <c r="F84" s="5">
-        <v>0</v>
-      </c>
-      <c r="H84" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E85" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="F85" s="5">
-        <v>0</v>
-      </c>
-      <c r="G85" s="5"/>
-      <c r="H85" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E86" s="5" t="s">
-        <v>128</v>
       </c>
       <c r="F86" s="5">
         <v>0</v>
       </c>
-      <c r="G86" s="5"/>
       <c r="H86" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="87" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E87" s="5" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F87" s="5">
         <v>0</v>
       </c>
+      <c r="G87" s="5"/>
       <c r="H87" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="88" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E88" s="5" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="F88" s="5">
         <v>0</v>
       </c>
+      <c r="G88" s="5"/>
       <c r="H88" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="89" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E89" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F89" s="5">
         <v>0</v>
@@ -2422,33 +2444,31 @@
         <v>73</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="90" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E90" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F90" s="5">
         <v>0</v>
       </c>
-      <c r="G90" s="5"/>
       <c r="H90" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="91" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E91" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F91" s="5">
         <v>0</v>
       </c>
-      <c r="G91" s="5"/>
       <c r="H91" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="92" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E92" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F92" s="5">
         <v>0</v>
@@ -2458,9 +2478,9 @@
         <v>73</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="93" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E93" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F93" s="5">
         <v>0</v>
@@ -2470,39 +2490,45 @@
         <v>73</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="94" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E94" s="5" t="s">
-        <v>200</v>
+        <v>138</v>
       </c>
       <c r="F94" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G94" s="5"/>
       <c r="H94" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F95" s="4"/>
-    </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A96" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="B96" s="1"/>
-      <c r="C96" s="1"/>
-      <c r="D96" s="1"/>
-      <c r="E96" s="2"/>
-      <c r="F96" s="2"/>
-      <c r="G96" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="H96" s="2"/>
-      <c r="I96" s="2"/>
+    <row r="95" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E95" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="F95" s="5">
+        <v>0</v>
+      </c>
+      <c r="G95" s="5"/>
+      <c r="H95" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="96" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E96" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="F96" s="5">
+        <v>0</v>
+      </c>
+      <c r="G96" s="5"/>
+      <c r="H96" s="5" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E97" s="5" t="s">
-        <v>107</v>
+        <v>207</v>
       </c>
       <c r="F97" s="5">
         <v>0</v>
@@ -2513,97 +2539,62 @@
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>42</v>
-      </c>
-      <c r="C98" t="s">
-        <v>11</v>
-      </c>
-      <c r="D98" t="s">
-        <v>44</v>
-      </c>
-      <c r="E98" t="s">
+      <c r="E98" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="F98" s="5">
+        <v>1</v>
+      </c>
+      <c r="G98" s="5"/>
+      <c r="H98" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F99" s="4"/>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A100" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B100" s="1"/>
+      <c r="C100" s="1"/>
+      <c r="D100" s="1"/>
+      <c r="E100" s="2"/>
+      <c r="F100" s="2"/>
+      <c r="G100" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="H100" s="2"/>
+      <c r="I100" s="2"/>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E101" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="F98">
-        <v>210</v>
-      </c>
-      <c r="I98" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>41</v>
-      </c>
-      <c r="C99" t="s">
-        <v>11</v>
-      </c>
-      <c r="D99" t="s">
-        <v>44</v>
-      </c>
-      <c r="E99" t="s">
-        <v>107</v>
-      </c>
-      <c r="F99" s="9">
-        <v>235</v>
-      </c>
-      <c r="I99" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>42</v>
-      </c>
-      <c r="C100" t="s">
-        <v>12</v>
-      </c>
-      <c r="D100" t="s">
-        <v>44</v>
-      </c>
-      <c r="E100" t="s">
-        <v>107</v>
-      </c>
-      <c r="F100" s="9">
-        <v>230</v>
-      </c>
-      <c r="I100" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>41</v>
-      </c>
-      <c r="C101" t="s">
-        <v>12</v>
-      </c>
-      <c r="D101" t="s">
-        <v>44</v>
-      </c>
-      <c r="E101" t="s">
-        <v>107</v>
-      </c>
-      <c r="F101" s="9">
-        <v>230</v>
-      </c>
-      <c r="I101" t="s">
-        <v>109</v>
+      <c r="F101" s="5">
+        <v>0</v>
+      </c>
+      <c r="G101" s="5"/>
+      <c r="H101" s="5" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>34</v>
+        <v>42</v>
+      </c>
+      <c r="C102" t="s">
+        <v>11</v>
       </c>
       <c r="D102" t="s">
-        <v>75</v>
+        <v>44</v>
       </c>
       <c r="E102" t="s">
         <v>107</v>
       </c>
-      <c r="F102" s="9">
-        <v>140</v>
+      <c r="F102">
+        <v>210</v>
       </c>
       <c r="I102" t="s">
         <v>108</v>
@@ -2611,16 +2602,19 @@
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>14</v>
+        <v>41</v>
+      </c>
+      <c r="C103" t="s">
+        <v>11</v>
       </c>
       <c r="D103" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="E103" t="s">
         <v>107</v>
       </c>
       <c r="F103" s="9">
-        <v>180</v>
+        <v>235</v>
       </c>
       <c r="I103" t="s">
         <v>108</v>
@@ -2628,79 +2622,73 @@
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="C104" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D104" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="E104" t="s">
         <v>107</v>
       </c>
       <c r="F104" s="9">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="I104" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="C105" t="s">
         <v>12</v>
       </c>
       <c r="D105" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="E105" t="s">
         <v>107</v>
       </c>
       <c r="F105" s="9">
-        <v>210</v>
-      </c>
-      <c r="H105" t="s">
-        <v>114</v>
+        <v>230</v>
+      </c>
+      <c r="I105" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>13</v>
-      </c>
-      <c r="C106" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="D106" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E106" t="s">
         <v>107</v>
       </c>
       <c r="F106" s="9">
-        <v>210</v>
+        <v>140</v>
       </c>
       <c r="I106" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>27</v>
-      </c>
-      <c r="C107" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D107" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E107" t="s">
         <v>107</v>
       </c>
       <c r="F107" s="9">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="I107" t="s">
         <v>108</v>
@@ -2708,685 +2696,729 @@
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="C108" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D108" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E108" t="s">
         <v>107</v>
       </c>
       <c r="F108" s="9">
-        <v>230</v>
+        <v>180</v>
       </c>
       <c r="I108" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>40</v>
+        <v>14</v>
+      </c>
+      <c r="C109" t="s">
+        <v>12</v>
       </c>
       <c r="D109" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="E109" t="s">
         <v>107</v>
       </c>
-      <c r="F109">
-        <v>180</v>
-      </c>
-      <c r="I109" t="s">
-        <v>108</v>
+      <c r="F109" s="9">
+        <v>210</v>
+      </c>
+      <c r="H109" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>39</v>
+        <v>13</v>
+      </c>
+      <c r="C110" t="s">
+        <v>12</v>
       </c>
       <c r="D110" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="E110" t="s">
         <v>107</v>
       </c>
-      <c r="F110">
-        <v>180</v>
-      </c>
-      <c r="H110" t="s">
-        <v>115</v>
+      <c r="F110" s="9">
+        <v>210</v>
+      </c>
+      <c r="I110" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A111" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B111" s="4"/>
+      <c r="A111" t="s">
+        <v>27</v>
+      </c>
+      <c r="C111" t="s">
+        <v>11</v>
+      </c>
+      <c r="D111" t="s">
+        <v>76</v>
+      </c>
+      <c r="E111" t="s">
+        <v>107</v>
+      </c>
+      <c r="F111" s="9">
+        <v>190</v>
+      </c>
+      <c r="I111" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A112" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B112" s="9"/>
-      <c r="C112" s="9"/>
-      <c r="D112" s="9" t="s">
+      <c r="A112" t="s">
+        <v>27</v>
+      </c>
+      <c r="C112" t="s">
+        <v>12</v>
+      </c>
+      <c r="D112" t="s">
         <v>76</v>
       </c>
       <c r="E112" t="s">
         <v>107</v>
       </c>
       <c r="F112" s="9">
-        <v>100</v>
+        <v>230</v>
       </c>
       <c r="I112" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A113" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B113" s="9"/>
-      <c r="C113" s="9"/>
-      <c r="D113" s="9" t="s">
-        <v>72</v>
+      <c r="A113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113" t="s">
+        <v>83</v>
       </c>
       <c r="E113" t="s">
         <v>107</v>
       </c>
-      <c r="F113" s="9">
-        <v>110</v>
+      <c r="F113">
+        <v>180</v>
+      </c>
+      <c r="I113" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A114" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="B114" s="5"/>
-      <c r="C114" s="5"/>
-      <c r="D114" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="E114" s="5" t="s">
+      <c r="A114" t="s">
+        <v>39</v>
+      </c>
+      <c r="D114" t="s">
+        <v>83</v>
+      </c>
+      <c r="E114" t="s">
         <v>107</v>
       </c>
-      <c r="F114" s="5">
-        <v>0</v>
-      </c>
-      <c r="G114" s="5"/>
-      <c r="H114" s="5" t="s">
-        <v>193</v>
+      <c r="F114">
+        <v>180</v>
+      </c>
+      <c r="H114" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>32</v>
-      </c>
-      <c r="C115" t="s">
-        <v>11</v>
-      </c>
-      <c r="D115" t="s">
-        <v>84</v>
-      </c>
-      <c r="E115" t="s">
-        <v>107</v>
-      </c>
-      <c r="F115">
-        <v>20</v>
-      </c>
-      <c r="H115" t="s">
-        <v>111</v>
-      </c>
-      <c r="I115" t="s">
-        <v>108</v>
-      </c>
+      <c r="A115" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B115" s="4"/>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
-        <v>32</v>
-      </c>
-      <c r="C116" t="s">
-        <v>12</v>
-      </c>
-      <c r="D116" t="s">
-        <v>84</v>
+      <c r="A116" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B116" s="9"/>
+      <c r="C116" s="9"/>
+      <c r="D116" s="9" t="s">
+        <v>76</v>
       </c>
       <c r="E116" t="s">
         <v>107</v>
       </c>
-      <c r="F116">
-        <v>21</v>
-      </c>
-      <c r="H116" t="s">
-        <v>111</v>
+      <c r="F116" s="9">
+        <v>100</v>
       </c>
       <c r="I116" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A117" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B117" s="4"/>
+      <c r="A117" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B117" s="9"/>
+      <c r="C117" s="9"/>
+      <c r="D117" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="E117" t="s">
+        <v>107</v>
+      </c>
+      <c r="F117" s="9">
+        <v>110</v>
+      </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>15</v>
-      </c>
-      <c r="C118" t="s">
-        <v>11</v>
-      </c>
-      <c r="D118" t="s">
-        <v>85</v>
-      </c>
-      <c r="E118" t="s">
+      <c r="A118" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B118" s="5"/>
+      <c r="C118" s="5"/>
+      <c r="D118" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E118" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="F118">
-        <v>9</v>
-      </c>
-      <c r="I118" t="s">
-        <v>108</v>
+      <c r="F118" s="5">
+        <v>0</v>
+      </c>
+      <c r="G118" s="5"/>
+      <c r="H118" s="5" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="C119" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D119" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E119" t="s">
         <v>107</v>
       </c>
       <c r="F119">
-        <v>9.5</v>
+        <v>20</v>
+      </c>
+      <c r="H119" t="s">
+        <v>111</v>
       </c>
       <c r="I119" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>32</v>
+      </c>
+      <c r="C120" t="s">
+        <v>12</v>
+      </c>
+      <c r="D120" t="s">
+        <v>84</v>
+      </c>
+      <c r="E120" t="s">
+        <v>107</v>
+      </c>
+      <c r="F120">
+        <v>21</v>
+      </c>
+      <c r="H120" t="s">
+        <v>111</v>
+      </c>
+      <c r="I120" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A120" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B120" s="4"/>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B121" s="4"/>
+    </row>
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>15</v>
+      </c>
+      <c r="C122" t="s">
+        <v>11</v>
+      </c>
+      <c r="D122" t="s">
+        <v>85</v>
+      </c>
+      <c r="E122" t="s">
+        <v>107</v>
+      </c>
+      <c r="F122">
+        <v>9</v>
+      </c>
+      <c r="I122" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>15</v>
+      </c>
+      <c r="C123" t="s">
+        <v>12</v>
+      </c>
+      <c r="D123" t="s">
+        <v>85</v>
+      </c>
+      <c r="E123" t="s">
+        <v>107</v>
+      </c>
+      <c r="F123">
+        <v>9.5</v>
+      </c>
+      <c r="I123" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A124" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B124" s="4"/>
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A125" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="B121" s="5"/>
-      <c r="C121" s="5"/>
-      <c r="D121" s="5"/>
-      <c r="E121" s="5"/>
-      <c r="F121" s="5"/>
-      <c r="G121" s="5"/>
-      <c r="H121" s="5"/>
-    </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A122" s="4" t="s">
+      <c r="B125" s="5"/>
+      <c r="C125" s="5"/>
+      <c r="D125" s="5"/>
+      <c r="E125" s="5"/>
+      <c r="F125" s="5"/>
+      <c r="G125" s="5"/>
+      <c r="H125" s="5"/>
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A126" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="B122" s="5"/>
-      <c r="C122" s="5"/>
-      <c r="D122" s="5"/>
-      <c r="E122" s="5"/>
-      <c r="F122" s="5"/>
-      <c r="G122" s="5"/>
-      <c r="H122" s="5"/>
-    </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A123" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="B123" s="5"/>
-      <c r="C123" s="5"/>
-      <c r="D123" s="5"/>
-      <c r="E123" s="5"/>
-      <c r="F123" s="5"/>
-      <c r="G123" s="5"/>
-      <c r="H123" s="5"/>
-    </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
-        <v>67</v>
-      </c>
-      <c r="C124" t="s">
-        <v>11</v>
-      </c>
-      <c r="D124" t="s">
-        <v>82</v>
-      </c>
-      <c r="E124" t="s">
-        <v>107</v>
-      </c>
-      <c r="F124">
-        <v>0.33</v>
-      </c>
-      <c r="I124" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
-        <v>67</v>
-      </c>
-      <c r="C125" t="s">
-        <v>12</v>
-      </c>
-      <c r="D125" t="s">
-        <v>82</v>
-      </c>
-      <c r="E125" t="s">
-        <v>107</v>
-      </c>
-      <c r="F125">
-        <f>(5+0.4)/2</f>
-        <v>2.7</v>
-      </c>
-      <c r="H125" t="s">
-        <v>110</v>
-      </c>
-      <c r="I125" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
-        <v>66</v>
-      </c>
-      <c r="D126" t="s">
-        <v>82</v>
-      </c>
-      <c r="E126" t="s">
-        <v>107</v>
-      </c>
-      <c r="F126">
-        <v>0.67</v>
-      </c>
-      <c r="I126" t="s">
-        <v>108</v>
-      </c>
+      <c r="B126" s="5"/>
+      <c r="C126" s="5"/>
+      <c r="D126" s="5"/>
+      <c r="E126" s="5"/>
+      <c r="F126" s="5"/>
+      <c r="G126" s="5"/>
+      <c r="H126" s="5"/>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" s="4" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B127" s="5"/>
       <c r="C127" s="5"/>
       <c r="D127" s="5"/>
       <c r="E127" s="5"/>
       <c r="F127" s="5"/>
+      <c r="G127" s="5"/>
+      <c r="H127" s="5"/>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A128" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="B128" s="5"/>
-      <c r="C128" s="5"/>
-      <c r="D128" s="5"/>
-      <c r="E128" s="5"/>
-      <c r="F128" s="5"/>
+      <c r="A128" t="s">
+        <v>67</v>
+      </c>
+      <c r="C128" t="s">
+        <v>11</v>
+      </c>
+      <c r="D128" t="s">
+        <v>82</v>
+      </c>
+      <c r="E128" t="s">
+        <v>107</v>
+      </c>
+      <c r="F128">
+        <v>0.33</v>
+      </c>
+      <c r="I128" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A129" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="B129" s="5"/>
-      <c r="C129" s="5"/>
-      <c r="D129" s="5"/>
-      <c r="E129" s="5"/>
-      <c r="F129" s="5"/>
+      <c r="A129" t="s">
+        <v>67</v>
+      </c>
+      <c r="C129" t="s">
+        <v>12</v>
+      </c>
+      <c r="D129" t="s">
+        <v>82</v>
+      </c>
+      <c r="E129" t="s">
+        <v>107</v>
+      </c>
+      <c r="F129">
+        <f>(5+0.4)/2</f>
+        <v>2.7</v>
+      </c>
+      <c r="H129" t="s">
+        <v>110</v>
+      </c>
+      <c r="I129" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D130" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E130" t="s">
         <v>107</v>
       </c>
       <c r="F130">
+        <v>0.67</v>
+      </c>
+      <c r="I130" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A131" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B131" s="5"/>
+      <c r="C131" s="5"/>
+      <c r="D131" s="5"/>
+      <c r="E131" s="5"/>
+      <c r="F131" s="5"/>
+    </row>
+    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A132" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B132" s="5"/>
+      <c r="C132" s="5"/>
+      <c r="D132" s="5"/>
+      <c r="E132" s="5"/>
+      <c r="F132" s="5"/>
+    </row>
+    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A133" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B133" s="5"/>
+      <c r="C133" s="5"/>
+      <c r="D133" s="5"/>
+      <c r="E133" s="5"/>
+      <c r="F133" s="5"/>
+    </row>
+    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>64</v>
+      </c>
+      <c r="D134" t="s">
+        <v>78</v>
+      </c>
+      <c r="E134" t="s">
+        <v>107</v>
+      </c>
+      <c r="F134">
         <f>900+1800</f>
         <v>2700</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A131" t="s">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
         <v>63</v>
       </c>
-      <c r="D131" t="s">
+      <c r="D135" t="s">
         <v>77</v>
       </c>
-      <c r="E131" t="s">
+      <c r="E135" t="s">
         <v>107</v>
       </c>
-      <c r="F131">
+      <c r="F135">
         <v>2000</v>
       </c>
-      <c r="H131" t="s">
+      <c r="H135" t="s">
         <v>112</v>
       </c>
-      <c r="I131" s="10" t="s">
+      <c r="I135" s="10" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A132" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B132" s="4"/>
-      <c r="H132" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A133" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B133" s="4"/>
-      <c r="D133" t="s">
-        <v>95</v>
-      </c>
-      <c r="E133" t="s">
-        <v>107</v>
-      </c>
-      <c r="F133" s="4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A134" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B134" s="4"/>
-    </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A135" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B135" s="4"/>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" s="4" t="s">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="B136" s="4"/>
+      <c r="H136" s="4" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" s="4" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B137" s="4"/>
+      <c r="D137" t="s">
+        <v>95</v>
+      </c>
+      <c r="E137" t="s">
+        <v>107</v>
+      </c>
+      <c r="F137" s="4">
+        <v>5</v>
+      </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A138" s="9" t="s">
-        <v>22</v>
+      <c r="A138" s="4" t="s">
+        <v>18</v>
       </c>
       <c r="B138" s="4"/>
-      <c r="D138" t="s">
-        <v>95</v>
-      </c>
-      <c r="E138" t="s">
-        <v>107</v>
-      </c>
-      <c r="F138">
-        <v>7</v>
-      </c>
-      <c r="H138" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="I138" t="s">
-        <v>108</v>
-      </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A139" s="9" t="s">
-        <v>23</v>
+      <c r="A139" s="4" t="s">
+        <v>53</v>
       </c>
       <c r="B139" s="4"/>
-      <c r="D139" t="s">
-        <v>95</v>
-      </c>
-      <c r="E139" t="s">
-        <v>107</v>
-      </c>
-      <c r="F139">
-        <v>4</v>
-      </c>
-      <c r="H139" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="I139" t="s">
-        <v>108</v>
-      </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="4" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="B140" s="4"/>
-      <c r="H140" s="4" t="s">
-        <v>118</v>
-      </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B141" s="4"/>
+    </row>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A142" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B142" s="4"/>
+      <c r="D142" t="s">
+        <v>95</v>
+      </c>
+      <c r="E142" t="s">
+        <v>107</v>
+      </c>
+      <c r="F142">
+        <v>7</v>
+      </c>
+      <c r="H142" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="I142" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A143" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B143" s="4"/>
+      <c r="D143" t="s">
+        <v>95</v>
+      </c>
+      <c r="E143" t="s">
+        <v>107</v>
+      </c>
+      <c r="F143">
+        <v>4</v>
+      </c>
+      <c r="H143" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="I143" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A144" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B144" s="4"/>
+      <c r="H144" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A145" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B141" s="4"/>
-    </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A142" s="4" t="s">
+      <c r="B145" s="4"/>
+    </row>
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A146" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B142" s="4"/>
-    </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A143" s="4" t="s">
+      <c r="B146" s="4"/>
+    </row>
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A147" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B143" s="4"/>
-    </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A144" s="9" t="s">
+      <c r="B147" s="4"/>
+    </row>
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A148" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B144" s="9"/>
-      <c r="C144" s="9"/>
-      <c r="D144" s="9"/>
-      <c r="E144" s="9"/>
-      <c r="F144" s="3">
+      <c r="B148" s="9"/>
+      <c r="C148" s="9"/>
+      <c r="D148" s="9"/>
+      <c r="E148" s="9"/>
+      <c r="F148" s="3">
         <v>0</v>
       </c>
-      <c r="H144" t="s">
+      <c r="H148" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A145" s="3" t="s">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A149" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="B145" s="9"/>
-      <c r="C145" s="9"/>
-      <c r="D145" s="9"/>
-      <c r="E145" s="9"/>
-      <c r="F145" s="3">
+      <c r="B149" s="9"/>
+      <c r="C149" s="9"/>
+      <c r="D149" s="9"/>
+      <c r="E149" s="9"/>
+      <c r="F149" s="3">
         <v>0</v>
       </c>
-      <c r="H145" t="s">
+      <c r="H149" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A146" s="3" t="s">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A150" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="B146" s="9"/>
-      <c r="C146" s="9"/>
-      <c r="D146" s="9"/>
-      <c r="E146" s="9"/>
-      <c r="F146" s="9">
+      <c r="B150" s="9"/>
+      <c r="C150" s="9"/>
+      <c r="D150" s="9"/>
+      <c r="E150" s="9"/>
+      <c r="F150" s="9">
         <v>0</v>
       </c>
-      <c r="H146" t="s">
+      <c r="H150" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A147" s="9" t="s">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A151" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B147" s="9"/>
-      <c r="C147" s="9"/>
-      <c r="D147" s="9"/>
-      <c r="E147" s="9"/>
-      <c r="F147" s="9">
+      <c r="B151" s="9"/>
+      <c r="C151" s="9"/>
+      <c r="D151" s="9"/>
+      <c r="E151" s="9"/>
+      <c r="F151" s="9">
         <v>0</v>
       </c>
-      <c r="H147" t="s">
+      <c r="H151" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A148" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B148" s="4"/>
-    </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A149" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B149" s="4"/>
-    </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A150" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B150" s="4"/>
-    </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A151" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B151" s="4"/>
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A152" s="4" t="s">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="B152" s="4"/>
     </row>
     <row r="153" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A153" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B153" s="4"/>
     </row>
     <row r="154" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A154" s="4" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B154" s="4"/>
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A155" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B155" s="4"/>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A156" s="4" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="B156" s="4"/>
     </row>
     <row r="157" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A157" s="4" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="B157" s="4"/>
     </row>
     <row r="158" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A158" s="4" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="B158" s="4"/>
     </row>
     <row r="159" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A159" s="4" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B159" s="4"/>
     </row>
     <row r="160" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A160" s="4" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="B160" s="4"/>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" s="4" t="s">
-        <v>62</v>
+        <v>37</v>
       </c>
       <c r="B161" s="4"/>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" s="4" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="B162" s="4"/>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A163" s="4" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="B163" s="4"/>
-      <c r="G163" s="4" t="s">
-        <v>164</v>
-      </c>
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" s="4" t="s">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="B164" s="4"/>
-      <c r="G164" s="4" t="s">
-        <v>164</v>
-      </c>
     </row>
     <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A165" s="4" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="B165" s="4"/>
-      <c r="G165" s="4" t="s">
-        <v>164</v>
-      </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A166" s="4" t="s">
-        <v>61</v>
+        <v>30</v>
       </c>
       <c r="B166" s="4"/>
-      <c r="G166" s="4" t="s">
-        <v>164</v>
-      </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A167" s="4" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="B167" s="4"/>
       <c r="G167" s="4" t="s">
@@ -3395,7 +3427,7 @@
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A168" s="4" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="B168" s="4"/>
       <c r="G168" s="4" t="s">
@@ -3404,7 +3436,7 @@
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A169" s="4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B169" s="4"/>
       <c r="G169" s="4" t="s">
@@ -3412,252 +3444,244 @@
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F170" s="4"/>
+      <c r="A170" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B170" s="4"/>
+      <c r="G170" s="4" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A171" s="1" t="s">
+      <c r="A171" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B171" s="4"/>
+      <c r="G171" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A172" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B172" s="4"/>
+      <c r="G172" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A173" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B173" s="4"/>
+      <c r="G173" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F174" s="4"/>
+    </row>
+    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A175" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B171" s="1"/>
-      <c r="C171" s="1"/>
-      <c r="D171" s="1"/>
-      <c r="E171" s="2"/>
-      <c r="F171" s="2"/>
-      <c r="G171" s="2"/>
-      <c r="H171" s="2"/>
-      <c r="I171" s="2"/>
-    </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B172" t="s">
+      <c r="B175" s="1"/>
+      <c r="C175" s="1"/>
+      <c r="D175" s="1"/>
+      <c r="E175" s="2"/>
+      <c r="F175" s="2"/>
+      <c r="G175" s="2"/>
+      <c r="H175" s="2"/>
+      <c r="I175" s="2"/>
+    </row>
+    <row r="176" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B176" t="s">
         <v>49</v>
       </c>
-      <c r="E172" t="s">
+      <c r="E176" t="s">
         <v>122</v>
       </c>
-      <c r="F172" s="11">
+      <c r="F176" s="11">
         <f>1/7*100</f>
         <v>14.285714285714285</v>
       </c>
-      <c r="G172" t="s">
+      <c r="G176" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B173" t="s">
+    <row r="177" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B177" t="s">
         <v>49</v>
       </c>
-      <c r="C173" t="s">
+      <c r="C177" t="s">
         <v>12</v>
       </c>
-      <c r="E173" t="s">
+      <c r="E177" t="s">
         <v>122</v>
       </c>
-      <c r="F173" s="4">
+      <c r="F177" s="4">
         <f>1/8*100</f>
         <v>12.5</v>
       </c>
-      <c r="G173" t="s">
+      <c r="G177" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B174" t="s">
+    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B178" t="s">
         <v>48</v>
       </c>
-      <c r="E174" t="s">
+      <c r="E178" t="s">
         <v>122</v>
       </c>
-      <c r="F174" s="11">
+      <c r="F178" s="11">
         <f>1/6*100</f>
         <v>16.666666666666664</v>
       </c>
-      <c r="G174" t="s">
+      <c r="G178" t="s">
         <v>123</v>
       </c>
-      <c r="I174" t="s">
+      <c r="I178" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B175" t="s">
+    <row r="179" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B179" t="s">
         <v>48</v>
       </c>
-      <c r="C175" t="s">
+      <c r="C179" t="s">
         <v>12</v>
       </c>
-      <c r="E175" t="s">
+      <c r="E179" t="s">
         <v>122</v>
       </c>
-      <c r="F175" s="11">
+      <c r="F179" s="11">
         <f>1/10*100</f>
         <v>10</v>
       </c>
-      <c r="G175" t="s">
+      <c r="G179" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F176" s="4"/>
-    </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A177" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="B177" s="1"/>
-      <c r="C177" s="1"/>
-      <c r="D177" s="1"/>
-      <c r="E177" s="2"/>
-      <c r="F177" s="2"/>
-      <c r="G177" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="H177" s="2"/>
-      <c r="I177" s="2"/>
-    </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E178" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F178" s="5">
-        <v>0</v>
-      </c>
-      <c r="G178" s="5"/>
-      <c r="H178" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="179" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E179" t="s">
-        <v>7</v>
-      </c>
-      <c r="F179" t="s">
-        <v>154</v>
-      </c>
-      <c r="H179" t="s">
-        <v>124</v>
-      </c>
-      <c r="I179" t="s">
-        <v>8</v>
-      </c>
+    <row r="180" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F180" s="4"/>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
-        <v>126</v>
+        <v>167</v>
       </c>
       <c r="B181" s="1"/>
       <c r="C181" s="1"/>
       <c r="D181" s="1"/>
       <c r="E181" s="2"/>
       <c r="F181" s="2"/>
-      <c r="G181" s="2"/>
+      <c r="G181" s="2" t="s">
+        <v>165</v>
+      </c>
       <c r="H181" s="2"/>
       <c r="I181" s="2"/>
     </row>
+    <row r="182" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E182" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F182" s="5">
+        <v>0</v>
+      </c>
+      <c r="G182" s="5"/>
+      <c r="H182" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A183" t="s">
-        <v>10</v>
-      </c>
       <c r="E183" t="s">
-        <v>125</v>
-      </c>
-      <c r="F183">
-        <v>1507</v>
-      </c>
-      <c r="G183" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="184" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A184" t="s">
-        <v>13</v>
-      </c>
-      <c r="E184" t="s">
-        <v>125</v>
-      </c>
-      <c r="F184">
-        <v>979</v>
+        <v>7</v>
+      </c>
+      <c r="F183" t="s">
+        <v>154</v>
+      </c>
+      <c r="H183" t="s">
+        <v>124</v>
+      </c>
+      <c r="I183" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A185" t="s">
-        <v>14</v>
-      </c>
-      <c r="E185" t="s">
-        <v>125</v>
-      </c>
-      <c r="F185">
-        <v>1211</v>
-      </c>
-    </row>
-    <row r="186" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A186" t="s">
-        <v>74</v>
-      </c>
-      <c r="E186" t="s">
-        <v>125</v>
-      </c>
-      <c r="F186">
-        <v>1779</v>
-      </c>
+      <c r="A185" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B185" s="1"/>
+      <c r="C185" s="1"/>
+      <c r="D185" s="1"/>
+      <c r="E185" s="2"/>
+      <c r="F185" s="2"/>
+      <c r="G185" s="2"/>
+      <c r="H185" s="2"/>
+      <c r="I185" s="2"/>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E187" t="s">
         <v>125</v>
       </c>
       <c r="F187">
-        <v>1092</v>
+        <v>1507</v>
+      </c>
+      <c r="G187" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="188" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E188" t="s">
         <v>125</v>
       </c>
       <c r="F188">
-        <v>1015</v>
+        <v>979</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="E189" t="s">
         <v>125</v>
       </c>
       <c r="F189">
-        <v>1015</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>17</v>
+        <v>74</v>
       </c>
       <c r="E190" t="s">
         <v>125</v>
       </c>
       <c r="F190">
-        <v>648</v>
+        <v>1779</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="E191" t="s">
         <v>125</v>
       </c>
       <c r="F191">
-        <v>1185</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="192" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>80</v>
+        <v>16</v>
       </c>
       <c r="E192" t="s">
         <v>125</v>
@@ -3668,255 +3692,255 @@
     </row>
     <row r="193" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E193" t="s">
         <v>125</v>
       </c>
       <c r="F193">
-        <v>944</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="194" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="E194" t="s">
         <v>125</v>
       </c>
       <c r="F194">
-        <v>628</v>
-      </c>
-      <c r="H194" t="s">
-        <v>205</v>
+        <v>648</v>
       </c>
     </row>
     <row r="195" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="E195" t="s">
         <v>125</v>
       </c>
       <c r="F195">
-        <v>628</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="196" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>19</v>
+        <v>80</v>
       </c>
       <c r="E196" t="s">
         <v>125</v>
       </c>
       <c r="F196">
-        <v>628</v>
-      </c>
-      <c r="H196" t="s">
-        <v>205</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="197" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="E197" t="s">
         <v>125</v>
       </c>
       <c r="F197">
-        <v>1185</v>
+        <v>944</v>
       </c>
     </row>
     <row r="198" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E198" t="s">
         <v>125</v>
       </c>
       <c r="F198">
-        <v>1092</v>
+        <v>628</v>
+      </c>
+      <c r="H198" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="199" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E199" t="s">
         <v>125</v>
       </c>
       <c r="F199">
-        <v>1015</v>
+        <v>628</v>
       </c>
     </row>
     <row r="200" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="E200" t="s">
         <v>125</v>
       </c>
       <c r="F200">
-        <v>1474</v>
+        <v>628</v>
+      </c>
+      <c r="H200" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="201" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E201" t="s">
         <v>125</v>
       </c>
       <c r="F201">
-        <v>628</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="202" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="E202" t="s">
         <v>125</v>
       </c>
       <c r="F202">
-        <v>628</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="203" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E203" t="s">
         <v>125</v>
       </c>
       <c r="F203">
-        <v>1073</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="204" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E204" t="s">
         <v>125</v>
       </c>
       <c r="F204">
-        <v>628</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="205" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E205" t="s">
         <v>125</v>
       </c>
       <c r="F205">
-        <v>1486</v>
+        <v>628</v>
       </c>
     </row>
     <row r="206" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E206" t="s">
         <v>125</v>
       </c>
       <c r="F206">
-        <v>1486</v>
+        <v>628</v>
       </c>
     </row>
     <row r="207" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E207" t="s">
         <v>125</v>
       </c>
       <c r="F207">
-        <v>648</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="208" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="E208" t="s">
         <v>125</v>
       </c>
       <c r="F208">
-        <v>979</v>
+        <v>628</v>
       </c>
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="E209" t="s">
         <v>125</v>
       </c>
       <c r="F209">
-        <v>1073</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="210" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E210" t="s">
         <v>125</v>
       </c>
       <c r="F210">
-        <v>944</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E211" t="s">
         <v>125</v>
       </c>
       <c r="F211">
-        <v>1015</v>
+        <v>648</v>
       </c>
     </row>
     <row r="212" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E212" t="s">
         <v>125</v>
       </c>
       <c r="F212">
-        <v>766</v>
+        <v>979</v>
       </c>
     </row>
     <row r="213" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="E213" t="s">
         <v>125</v>
       </c>
       <c r="F213">
-        <v>1507</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="214" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="E214" t="s">
         <v>125</v>
       </c>
       <c r="F214">
-        <v>1015</v>
+        <v>944</v>
       </c>
     </row>
     <row r="215" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="E215" t="s">
         <v>125</v>
@@ -3927,18 +3951,18 @@
     </row>
     <row r="216" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="E216" t="s">
         <v>125</v>
       </c>
       <c r="F216">
-        <v>1185</v>
+        <v>766</v>
       </c>
     </row>
     <row r="217" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="E217" t="s">
         <v>125</v>
@@ -3949,227 +3973,227 @@
     </row>
     <row r="218" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="E218" t="s">
         <v>125</v>
       </c>
       <c r="F218">
-        <v>1211</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E219" t="s">
         <v>125</v>
       </c>
       <c r="F219">
-        <v>1569</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="220" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E220" t="s">
         <v>125</v>
       </c>
       <c r="F220">
-        <v>1569</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="221" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E221" t="s">
         <v>125</v>
       </c>
       <c r="F221">
-        <v>766</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="222" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="E222" t="s">
         <v>125</v>
       </c>
       <c r="F222">
-        <v>1185</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="223" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="E223" t="s">
         <v>125</v>
       </c>
       <c r="F223">
-        <v>1015</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="224" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
+        <v>63</v>
+      </c>
+      <c r="E224" t="s">
+        <v>125</v>
+      </c>
+      <c r="F224">
+        <v>1569</v>
+      </c>
+    </row>
+    <row r="225" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
+        <v>64</v>
+      </c>
+      <c r="E225" t="s">
+        <v>125</v>
+      </c>
+      <c r="F225">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="226" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A226" t="s">
+        <v>65</v>
+      </c>
+      <c r="E226" t="s">
+        <v>125</v>
+      </c>
+      <c r="F226">
+        <v>1185</v>
+      </c>
+    </row>
+    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A227" t="s">
+        <v>66</v>
+      </c>
+      <c r="E227" t="s">
+        <v>125</v>
+      </c>
+      <c r="F227">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A228" t="s">
         <v>67</v>
       </c>
-      <c r="E224" t="s">
-        <v>125</v>
-      </c>
-      <c r="F224">
+      <c r="E228" t="s">
+        <v>125</v>
+      </c>
+      <c r="F228">
         <v>1211</v>
       </c>
     </row>
-    <row r="225" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A225" t="s">
+    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A229" t="s">
         <v>34</v>
       </c>
-      <c r="E225" t="s">
-        <v>125</v>
-      </c>
-      <c r="F225">
+      <c r="E229" t="s">
+        <v>125</v>
+      </c>
+      <c r="F229">
         <v>1015</v>
       </c>
     </row>
-    <row r="226" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A226" t="s">
+    <row r="230" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A230" t="s">
         <v>35</v>
       </c>
-      <c r="E226" t="s">
-        <v>125</v>
-      </c>
-      <c r="F226">
+      <c r="E230" t="s">
+        <v>125</v>
+      </c>
+      <c r="F230">
         <v>628</v>
       </c>
     </row>
-    <row r="227" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A227" t="s">
+    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A231" t="s">
         <v>36</v>
       </c>
-      <c r="E227" t="s">
-        <v>125</v>
-      </c>
-      <c r="F227">
+      <c r="E231" t="s">
+        <v>125</v>
+      </c>
+      <c r="F231">
         <v>628</v>
       </c>
     </row>
-    <row r="228" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A228" s="3" t="s">
+    <row r="232" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A232" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="E228" t="s">
-        <v>125</v>
-      </c>
-      <c r="F228">
+      <c r="E232" t="s">
+        <v>125</v>
+      </c>
+      <c r="F232">
         <v>628</v>
       </c>
     </row>
-    <row r="229" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A229" s="3" t="s">
+    <row r="233" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A233" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="E229" t="s">
-        <v>125</v>
-      </c>
-      <c r="F229">
+      <c r="E233" t="s">
+        <v>125</v>
+      </c>
+      <c r="F233">
         <v>628</v>
       </c>
     </row>
-    <row r="230" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A230" t="s">
+    <row r="234" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A234" t="s">
         <v>68</v>
       </c>
-      <c r="E230" t="s">
-        <v>125</v>
-      </c>
-      <c r="F230">
+      <c r="E234" t="s">
+        <v>125</v>
+      </c>
+      <c r="F234">
         <v>1224</v>
       </c>
     </row>
-    <row r="231" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A231" t="s">
+    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A235" t="s">
         <v>37</v>
       </c>
-      <c r="E231" t="s">
-        <v>125</v>
-      </c>
-      <c r="F231">
+      <c r="E235" t="s">
+        <v>125</v>
+      </c>
+      <c r="F235">
         <v>1015</v>
       </c>
     </row>
-    <row r="232" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A232" t="s">
+    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A236" t="s">
         <v>69</v>
       </c>
-      <c r="E232" t="s">
-        <v>125</v>
-      </c>
-      <c r="F232">
+      <c r="E236" t="s">
+        <v>125</v>
+      </c>
+      <c r="F236">
         <v>1015</v>
       </c>
     </row>
-    <row r="233" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A233" t="s">
+    <row r="237" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A237" t="s">
         <v>38</v>
       </c>
-      <c r="E233" t="s">
-        <v>125</v>
-      </c>
-      <c r="F233">
+      <c r="E237" t="s">
+        <v>125</v>
+      </c>
+      <c r="F237">
         <v>1721</v>
       </c>
     </row>
-    <row r="234" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A234" t="s">
+    <row r="238" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A238" t="s">
         <v>70</v>
-      </c>
-      <c r="E234" t="s">
-        <v>125</v>
-      </c>
-      <c r="F234">
-        <v>1015</v>
-      </c>
-    </row>
-    <row r="235" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A235" t="s">
-        <v>39</v>
-      </c>
-      <c r="E235" t="s">
-        <v>125</v>
-      </c>
-      <c r="F235">
-        <v>1211</v>
-      </c>
-    </row>
-    <row r="236" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A236" t="s">
-        <v>40</v>
-      </c>
-      <c r="E236" t="s">
-        <v>125</v>
-      </c>
-      <c r="F236">
-        <v>1211</v>
-      </c>
-    </row>
-    <row r="237" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A237" t="s">
-        <v>41</v>
-      </c>
-      <c r="E237" t="s">
-        <v>125</v>
-      </c>
-      <c r="F237">
-        <v>979</v>
-      </c>
-    </row>
-    <row r="238" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A238" t="s">
-        <v>42</v>
       </c>
       <c r="E238" t="s">
         <v>125</v>
@@ -4178,83 +4202,53 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="239" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A239" s="9" t="s">
+    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A239" t="s">
+        <v>39</v>
+      </c>
+      <c r="E239" t="s">
+        <v>125</v>
+      </c>
+      <c r="F239">
+        <v>1211</v>
+      </c>
+    </row>
+    <row r="240" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A240" t="s">
+        <v>40</v>
+      </c>
+      <c r="E240" t="s">
+        <v>125</v>
+      </c>
+      <c r="F240">
+        <v>1211</v>
+      </c>
+    </row>
+    <row r="241" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A241" t="s">
+        <v>41</v>
+      </c>
+      <c r="E241" t="s">
+        <v>125</v>
+      </c>
+      <c r="F241">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="242" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A242" t="s">
+        <v>42</v>
+      </c>
+      <c r="E242" t="s">
+        <v>125</v>
+      </c>
+      <c r="F242">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="243" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A243" s="9" t="s">
         <v>173</v>
-      </c>
-      <c r="B239" s="9"/>
-      <c r="C239" s="9"/>
-      <c r="D239" s="9"/>
-      <c r="E239" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="F239" s="9">
-        <v>1212</v>
-      </c>
-      <c r="G239" s="9"/>
-      <c r="H239" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="I239" s="5"/>
-    </row>
-    <row r="240" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A240" s="9" t="s">
-        <v>175</v>
-      </c>
-      <c r="B240" s="9"/>
-      <c r="C240" s="9"/>
-      <c r="D240" s="9"/>
-      <c r="E240" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="F240" s="9">
-        <v>1212</v>
-      </c>
-      <c r="G240" s="9"/>
-      <c r="H240" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="I240" s="5"/>
-    </row>
-    <row r="241" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A241" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="B241" s="9"/>
-      <c r="C241" s="9"/>
-      <c r="D241" s="9"/>
-      <c r="E241" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="F241" s="9">
-        <v>1212</v>
-      </c>
-      <c r="G241" s="9"/>
-      <c r="H241" s="9" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="242" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A242" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="B242" s="9"/>
-      <c r="C242" s="9"/>
-      <c r="D242" s="9"/>
-      <c r="E242" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="F242" s="9">
-        <v>1212</v>
-      </c>
-      <c r="G242" s="9"/>
-      <c r="H242" s="9" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="243" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A243" s="9" t="s">
-        <v>185</v>
       </c>
       <c r="B243" s="9"/>
       <c r="C243" s="9"/>
@@ -4263,16 +4257,17 @@
         <v>125</v>
       </c>
       <c r="F243" s="9">
-        <v>1779</v>
+        <v>1212</v>
       </c>
       <c r="G243" s="9"/>
       <c r="H243" s="9" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="244" spans="1:8" x14ac:dyDescent="0.25">
+        <v>174</v>
+      </c>
+      <c r="I243" s="5"/>
+    </row>
+    <row r="244" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A244" s="9" t="s">
-        <v>189</v>
+        <v>175</v>
       </c>
       <c r="B244" s="9"/>
       <c r="C244" s="9"/>
@@ -4285,12 +4280,13 @@
       </c>
       <c r="G244" s="9"/>
       <c r="H244" s="9" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="245" spans="1:8" x14ac:dyDescent="0.25">
+        <v>174</v>
+      </c>
+      <c r="I244" s="5"/>
+    </row>
+    <row r="245" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A245" s="9" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="B245" s="9"/>
       <c r="C245" s="9"/>
@@ -4299,24 +4295,96 @@
         <v>125</v>
       </c>
       <c r="F245" s="9">
-        <v>1779</v>
+        <v>1212</v>
       </c>
       <c r="G245" s="9"/>
       <c r="H245" s="9" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="246" spans="1:8" x14ac:dyDescent="0.25">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="246" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A246" s="9" t="s">
-        <v>199</v>
-      </c>
+        <v>187</v>
+      </c>
+      <c r="B246" s="9"/>
+      <c r="C246" s="9"/>
+      <c r="D246" s="9"/>
       <c r="E246" s="9" t="s">
         <v>125</v>
       </c>
       <c r="F246" s="9">
         <v>1212</v>
       </c>
+      <c r="G246" s="9"/>
       <c r="H246" s="9" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="247" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A247" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="B247" s="9"/>
+      <c r="C247" s="9"/>
+      <c r="D247" s="9"/>
+      <c r="E247" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="F247" s="9">
+        <v>1779</v>
+      </c>
+      <c r="G247" s="9"/>
+      <c r="H247" s="9" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="248" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A248" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="B248" s="9"/>
+      <c r="C248" s="9"/>
+      <c r="D248" s="9"/>
+      <c r="E248" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="F248" s="9">
+        <v>1212</v>
+      </c>
+      <c r="G248" s="9"/>
+      <c r="H248" s="9" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="249" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A249" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="B249" s="9"/>
+      <c r="C249" s="9"/>
+      <c r="D249" s="9"/>
+      <c r="E249" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="F249" s="9">
+        <v>1779</v>
+      </c>
+      <c r="G249" s="9"/>
+      <c r="H249" s="9" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="250" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A250" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="E250" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="F250" s="9">
+        <v>1212</v>
+      </c>
+      <c r="H250" s="9" t="s">
         <v>194</v>
       </c>
     </row>
@@ -4326,7 +4394,7 @@
     <sortCondition ref="C14:C9129"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="I131" r:id="rId1"/>
+    <hyperlink ref="I135" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>

</xml_diff>

<commit_message>
Updated crop residue C content and moved to main .xlsx file
</commit_message>
<xml_diff>
--- a/data/default/CropProduction.xlsx
+++ b/data/default/CropProduction.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5EB4B97-E071-4D36-A899-9FDA52FF7E27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF3A4FE-2EAF-44CE-8E59-0FBF152C2B9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25425" yWindow="4035" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3570" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="216">
   <si>
     <t>f_crop</t>
   </si>
@@ -658,9 +658,6 @@
     <t>frac_renew</t>
   </si>
   <si>
-    <t>Fraction of below ground residues renewed annually</t>
-  </si>
-  <si>
     <t>No prod., harvest = potential, assumed as organic ley * 0.5 need to check!!!</t>
   </si>
   <si>
@@ -701,6 +698,12 @@
   </si>
   <si>
     <t>Bolinder et al. 2007</t>
+  </si>
+  <si>
+    <t>Fraction of above and below ground residues renewed annually</t>
+  </si>
+  <si>
+    <t>Bolinder et al. (2007). An approach for estimating net primary productivity and annual carbon inputs to soil for common agricultural crops in Canada. Agriculture, Ecosystems &amp; Environment, 118(1), 29-42. https://doi.org/10.1016/j.agee.2006.05.013</t>
   </si>
 </sst>
 </file>
@@ -2150,7 +2153,7 @@
         <v>0</v>
       </c>
       <c r="H64" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -2165,7 +2168,7 @@
         <v>0</v>
       </c>
       <c r="H65" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -2180,7 +2183,7 @@
         <v>0</v>
       </c>
       <c r="H66" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -2264,7 +2267,7 @@
         <v>130</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="I75" s="3" t="s">
         <v>158</v>
@@ -2272,19 +2275,19 @@
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E76" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F76">
         <v>0.65</v>
       </c>
       <c r="G76" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H76" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="H76" s="3" t="s">
+      <c r="I76" s="3" t="s">
         <v>213</v>
-      </c>
-      <c r="I76" s="3" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -2376,16 +2379,19 @@
     </row>
     <row r="83" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E83" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="F83" t="s">
-        <v>152</v>
+        <v>204</v>
+      </c>
+      <c r="F83">
+        <v>0.45</v>
       </c>
       <c r="G83" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="H83" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="H83" s="3" t="s">
-        <v>208</v>
+      <c r="I83" s="3" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="84" spans="5:9" x14ac:dyDescent="0.25">
@@ -2407,18 +2413,20 @@
     </row>
     <row r="85" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E85" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="F85">
+        <v>0.45</v>
+      </c>
+      <c r="G85" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="F85" t="s">
-        <v>152</v>
-      </c>
-      <c r="G85" s="3" t="s">
-        <v>207</v>
-      </c>
       <c r="H85" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="I85" s="3"/>
+        <v>208</v>
+      </c>
+      <c r="I85" s="3" t="s">
+        <v>213</v>
+      </c>
     </row>
     <row r="86" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E86" s="3" t="s">
@@ -2429,7 +2437,7 @@
       </c>
       <c r="G86" s="3"/>
       <c r="H86" s="3" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="I86" s="3" t="s">
         <v>161</v>
@@ -2541,7 +2549,7 @@
     </row>
     <row r="96" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E96" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F96" s="5">
         <v>0</v>
@@ -2565,7 +2573,7 @@
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E98" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F98" s="5">
         <v>0</v>
@@ -3793,7 +3801,7 @@
         <v>628</v>
       </c>
       <c r="H199" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="200" spans="1:8" x14ac:dyDescent="0.25">
@@ -3818,7 +3826,7 @@
         <v>628</v>
       </c>
       <c r="H201" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="202" spans="1:8" x14ac:dyDescent="0.25">
@@ -4440,7 +4448,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -4463,6 +4471,11 @@
         <v>175</v>
       </c>
     </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>215</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>